<commit_message>
Add waterfall charts and mini-sparklines to 7 premium tools
Each cockpit now includes stacked-bar waterfalls (cash/MRR/pricing
bridges) plus unicode and line mini-sparklines for trend at a glance.
</commit_message>
<xml_diff>
--- a/public/planilhas/01_diagnostico_financeiro_360.xlsx
+++ b/public/planilhas/01_diagnostico_financeiro_360.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PROJECAO" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'DASHBOARD'!$A$1:$L$44</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'DASHBOARD'!$A$1:$R$60</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -21,13 +21,15 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="dd/mm"/>
     <numFmt numFmtId="166" formatCode="&quot;R$&quot; #,##0"/>
     <numFmt numFmtId="167" formatCode="0.0%"/>
+    <numFmt numFmtId="168" formatCode="#,##0;(#,##0);&quot;—&quot;"/>
+    <numFmt numFmtId="169" formatCode="#,##0.0;(#,##0.0);&quot;—&quot;"/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="26">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -95,7 +97,7 @@
     <font>
       <name val="Aptos Narrow"/>
       <color rgb="000E1512"/>
-      <sz val="9"/>
+      <sz val="8"/>
     </font>
     <font>
       <name val="Aptos Narrow"/>
@@ -129,11 +131,6 @@
     </font>
     <font>
       <name val="Aptos Narrow"/>
-      <color rgb="000E1512"/>
-      <sz val="8"/>
-    </font>
-    <font>
-      <name val="Aptos Narrow"/>
       <color rgb="00F3ECDD"/>
       <sz val="9"/>
     </font>
@@ -146,6 +143,37 @@
       <name val="Aptos Narrow"/>
       <color rgb="00C99C66"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <color rgb="008A9691"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <color rgb="008A9691"/>
+      <sz val="7"/>
+    </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <color rgb="0043D07F"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <color rgb="00C99C66"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <b val="1"/>
+      <color rgb="008A9691"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <color rgb="0043D07F"/>
+      <sz val="8"/>
     </font>
   </fonts>
   <fills count="5">
@@ -197,7 +225,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -235,19 +263,34 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="18" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="19" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="20" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="11" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="17" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="18" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="19" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="21" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="20" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="23" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -263,7 +306,23 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="3">
+    <dxf>
+      <font>
+        <name val="Aptos Narrow"/>
+        <b val="1"/>
+        <color rgb="0043D07F"/>
+        <sz val="9"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Aptos Narrow"/>
+        <b val="1"/>
+        <color rgb="00D9534F"/>
+        <sz val="9"/>
+      </font>
+    </dxf>
     <dxf>
       <font>
         <name val="Aptos Narrow"/>
@@ -500,6 +559,219 @@
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Cascata do mês</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="stacked"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'DASHBOARD'!O37</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'DASHBOARD'!$N$38:$N$40</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'DASHBOARD'!$O$38:$O$40</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'DASHBOARD'!P37</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="2E9E5B"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'DASHBOARD'!$N$38:$N$40</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'DASHBOARD'!$P$38:$P$40</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'DASHBOARD'!Q37</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="D9534F"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'DASHBOARD'!$N$38:$N$40</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'DASHBOARD'!$Q$38:$Q$40</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <overlap val="100"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="b"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="2"/>
+  <chart>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'DASHBOARD'!O49</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="15000">
+              <a:solidFill>
+                <a:srgbClr val="C99C66"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'DASHBOARD'!$N$50:$N$61</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'DASHBOARD'!$O$50:$O$61</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="2"/>
   <chart>
     <title>
@@ -628,6 +900,50 @@
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>35</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3960000" cy="2340000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="3" name="Chart 3"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>47</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3600000" cy="1620000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="4" name="Chart 4"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -952,7 +1268,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L60"/>
+  <dimension ref="A1:Z61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1074,27 +1390,27 @@
     <row r="6" ht="26" customHeight="1">
       <c r="A6" s="2" t="n"/>
       <c r="B6" s="7">
-        <f>B40</f>
+        <f>Z40</f>
         <v/>
       </c>
       <c r="C6" s="6" t="n"/>
       <c r="D6" s="8">
-        <f>B41</f>
+        <f>Z41</f>
         <v/>
       </c>
       <c r="E6" s="6" t="n"/>
       <c r="F6" s="9">
-        <f>B42</f>
+        <f>Z42</f>
         <v/>
       </c>
       <c r="G6" s="6" t="n"/>
       <c r="H6" s="10">
-        <f>B43</f>
+        <f>Z43</f>
         <v/>
       </c>
       <c r="I6" s="6" t="n"/>
       <c r="J6" s="11">
-        <f>B47</f>
+        <f>Z47</f>
         <v/>
       </c>
       <c r="K6" s="6" t="n"/>
@@ -1139,7 +1455,7 @@
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="2" t="n"/>
       <c r="B9" s="13">
-        <f>IF(B47&gt;=80,"🟢 Excelente — patrimônio crescendo. Mantenha os aportes.",IF(B47&gt;=60,"🟡 Saudável — reduza estilo de vida e aumente aportes.",IF(B47&gt;=40,"🟠 Atenção — controle gastos e comece a investir.","🔴 Crítico — corte dívidas e despesas não essenciais já.")))</f>
+        <f>IF(Z47&gt;=80,"🟢 Excelente — patrimônio crescendo. Mantenha os aportes.",IF(Z47&gt;=60,"🟡 Saudável — reduza estilo de vida e aumente aportes.",IF(Z47&gt;=40,"🟠 Atenção — controle gastos e comece a investir.","🔴 Crítico — corte dívidas e despesas não essenciais já.")))</f>
         <v/>
       </c>
       <c r="C9" s="14" t="n"/>
@@ -1157,7 +1473,7 @@
       <c r="A10" s="2" t="n"/>
       <c r="B10" s="2" t="n"/>
       <c r="C10" s="15">
-        <f>MAX(0,B42)</f>
+        <f>MAX(0,Z42)</f>
         <v/>
       </c>
       <c r="D10" s="2" t="n"/>
@@ -1240,7 +1556,7 @@
         <v/>
       </c>
       <c r="D14" s="20">
-        <f>IFERROR(C14/$B$40,0)</f>
+        <f>IFERROR(C14/$Z$40,0)</f>
         <v/>
       </c>
       <c r="E14" s="2" t="n"/>
@@ -1264,7 +1580,7 @@
         <v/>
       </c>
       <c r="D15" s="20">
-        <f>IFERROR(C15/$B$40,0)</f>
+        <f>IFERROR(C15/$Z$40,0)</f>
         <v/>
       </c>
       <c r="E15" s="2" t="n"/>
@@ -1288,7 +1604,7 @@
         <v/>
       </c>
       <c r="D16" s="20">
-        <f>IFERROR(C16/$B$40,0)</f>
+        <f>IFERROR(C16/$Z$40,0)</f>
         <v/>
       </c>
       <c r="E16" s="2" t="n"/>
@@ -1312,7 +1628,7 @@
         <v/>
       </c>
       <c r="D17" s="20">
-        <f>IFERROR(C17/$B$40,0)</f>
+        <f>IFERROR(C17/$Z$40,0)</f>
         <v/>
       </c>
       <c r="E17" s="2" t="n"/>
@@ -1336,7 +1652,7 @@
         <v/>
       </c>
       <c r="D18" s="20">
-        <f>IFERROR(C18/$B$40,0)</f>
+        <f>IFERROR(C18/$Z$40,0)</f>
         <v/>
       </c>
       <c r="E18" s="2" t="n"/>
@@ -1360,7 +1676,7 @@
         <v/>
       </c>
       <c r="D19" s="20">
-        <f>IFERROR(C19/$B$40,0)</f>
+        <f>IFERROR(C19/$Z$40,0)</f>
         <v/>
       </c>
       <c r="E19" s="2" t="n"/>
@@ -1384,7 +1700,7 @@
         <v/>
       </c>
       <c r="D20" s="20">
-        <f>IFERROR(C20/$B$40,0)</f>
+        <f>IFERROR(C20/$Z$40,0)</f>
         <v/>
       </c>
       <c r="E20" s="2" t="n"/>
@@ -1408,7 +1724,7 @@
         <v/>
       </c>
       <c r="D21" s="20">
-        <f>IFERROR(C21/$B$40,0)</f>
+        <f>IFERROR(C21/$Z$40,0)</f>
         <v/>
       </c>
       <c r="E21" s="2" t="n"/>
@@ -1432,7 +1748,7 @@
         <v/>
       </c>
       <c r="D22" s="20">
-        <f>IFERROR(C22/$B$40,0)</f>
+        <f>IFERROR(C22/$Z$40,0)</f>
         <v/>
       </c>
       <c r="E22" s="2" t="n"/>
@@ -1456,7 +1772,7 @@
         <v/>
       </c>
       <c r="D23" s="20">
-        <f>IFERROR(C23/$B$40,0)</f>
+        <f>IFERROR(C23/$Z$40,0)</f>
         <v/>
       </c>
       <c r="E23" s="2" t="n"/>
@@ -1548,7 +1864,7 @@
         </is>
       </c>
       <c r="G28" s="22">
-        <f>MIN(100,MAX(0,B43)*400)</f>
+        <f>MIN(100,MAX(0,Z43)*400)</f>
         <v/>
       </c>
       <c r="H28" s="2" t="n"/>
@@ -1569,7 +1885,7 @@
         </is>
       </c>
       <c r="G29" s="22">
-        <f>MIN(100,IFERROR(B44/B40,0)*400)</f>
+        <f>MIN(100,IFERROR(Z44/Z40,0)*400)</f>
         <v/>
       </c>
       <c r="H29" s="2" t="n"/>
@@ -1590,7 +1906,7 @@
         </is>
       </c>
       <c r="G30" s="22">
-        <f>MAX(0,100-(B46-0.5)*120)</f>
+        <f>MAX(0,100-(Z46-0.5)*120)</f>
         <v/>
       </c>
       <c r="H30" s="2" t="n"/>
@@ -1611,7 +1927,7 @@
         </is>
       </c>
       <c r="G31" s="22">
-        <f>MAX(0,100-IFERROR(B45/B40,0)*300)</f>
+        <f>MAX(0,100-IFERROR(Z45/Z40,0)*300)</f>
         <v/>
       </c>
       <c r="H31" s="2" t="n"/>
@@ -1632,7 +1948,7 @@
         </is>
       </c>
       <c r="G32" s="22">
-        <f>MIN(100,IFERROR(B42/B41,0)*100)</f>
+        <f>MIN(100,IFERROR(Z42/Z41,0)*100)</f>
         <v/>
       </c>
       <c r="H32" s="2" t="n"/>
@@ -1685,7 +2001,11 @@
     </row>
     <row r="36">
       <c r="A36" s="2" t="n"/>
-      <c r="B36" s="2" t="n"/>
+      <c r="B36" s="16" t="inlineStr">
+        <is>
+          <t>MINI-SPARKLINES</t>
+        </is>
+      </c>
       <c r="C36" s="2" t="n"/>
       <c r="D36" s="2" t="n"/>
       <c r="E36" s="2" t="n"/>
@@ -1696,89 +2016,324 @@
       <c r="J36" s="2" t="n"/>
       <c r="K36" s="2" t="n"/>
       <c r="L36" s="2" t="n"/>
-    </row>
-    <row r="37">
+      <c r="N36" s="23" t="inlineStr">
+        <is>
+          <t>Cascata Renda → Saldo</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="26" customHeight="1">
       <c r="A37" s="2" t="n"/>
-      <c r="B37" s="2" t="n"/>
-      <c r="C37" s="2" t="n"/>
-      <c r="D37" s="2" t="n"/>
-      <c r="E37" s="2" t="n"/>
-      <c r="F37" s="2" t="n"/>
-      <c r="G37" s="2" t="n"/>
-      <c r="H37" s="2" t="n"/>
-      <c r="I37" s="2" t="n"/>
-      <c r="J37" s="2" t="n"/>
+      <c r="B37" s="17" t="inlineStr">
+        <is>
+          <t>Indicador</t>
+        </is>
+      </c>
+      <c r="C37" s="17" t="inlineStr">
+        <is>
+          <t>Atual</t>
+        </is>
+      </c>
+      <c r="D37" s="17" t="inlineStr">
+        <is>
+          <t>S1</t>
+        </is>
+      </c>
+      <c r="E37" s="17" t="inlineStr">
+        <is>
+          <t>S2</t>
+        </is>
+      </c>
+      <c r="F37" s="17" t="inlineStr">
+        <is>
+          <t>S3</t>
+        </is>
+      </c>
+      <c r="G37" s="17" t="inlineStr">
+        <is>
+          <t>S4</t>
+        </is>
+      </c>
+      <c r="H37" s="17" t="inlineStr">
+        <is>
+          <t>S5</t>
+        </is>
+      </c>
+      <c r="I37" s="17" t="inlineStr">
+        <is>
+          <t>S6</t>
+        </is>
+      </c>
+      <c r="J37" s="17" t="inlineStr">
+        <is>
+          <t>Spark</t>
+        </is>
+      </c>
       <c r="K37" s="2" t="n"/>
       <c r="L37" s="2" t="n"/>
+      <c r="N37" s="17" t="inlineStr">
+        <is>
+          <t>Etapa</t>
+        </is>
+      </c>
+      <c r="O37" s="17" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="P37" s="17" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="Q37" s="17" t="inlineStr">
+        <is>
+          <t>Baixa</t>
+        </is>
+      </c>
+      <c r="R37" s="17" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="S37" s="17" t="inlineStr">
+        <is>
+          <t>Δ</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n"/>
-      <c r="B38" s="2" t="n"/>
-      <c r="C38" s="2" t="n"/>
-      <c r="D38" s="2" t="n"/>
-      <c r="E38" s="2" t="n"/>
-      <c r="F38" s="2" t="n"/>
-      <c r="G38" s="2" t="n"/>
-      <c r="H38" s="2" t="n"/>
-      <c r="I38" s="2" t="n"/>
-      <c r="J38" s="2" t="n"/>
+      <c r="B38" s="18" t="inlineStr">
+        <is>
+          <t>Poupança %</t>
+        </is>
+      </c>
+      <c r="C38" s="24">
+        <f>$Z$43*100</f>
+        <v/>
+      </c>
+      <c r="D38" s="25" t="n">
+        <v>10</v>
+      </c>
+      <c r="E38" s="25" t="n">
+        <v>12</v>
+      </c>
+      <c r="F38" s="25" t="n">
+        <v>15</v>
+      </c>
+      <c r="G38" s="25" t="n">
+        <v>18</v>
+      </c>
+      <c r="H38" s="25" t="n">
+        <v>22</v>
+      </c>
+      <c r="I38" s="25">
+        <f>$Z$43*100</f>
+        <v/>
+      </c>
+      <c r="J38" s="26">
+        <f>IF(D38=""," ",MID("▁▂▃▄▅▆▇█",MAX(1,MIN(8,ROUND((D38-(MIN(D38:I38)))/MAX(1E-9,(MAX(D38:I38))-(MIN(D38:I38)))*7+1,0))),1))&amp;IF(E38=""," ",MID("▁▂▃▄▅▆▇█",MAX(1,MIN(8,ROUND((E38-(MIN(D38:I38)))/MAX(1E-9,(MAX(D38:I38))-(MIN(D38:I38)))*7+1,0))),1))&amp;IF(F38=""," ",MID("▁▂▃▄▅▆▇█",MAX(1,MIN(8,ROUND((F38-(MIN(D38:I38)))/MAX(1E-9,(MAX(D38:I38))-(MIN(D38:I38)))*7+1,0))),1))&amp;IF(G38=""," ",MID("▁▂▃▄▅▆▇█",MAX(1,MIN(8,ROUND((G38-(MIN(D38:I38)))/MAX(1E-9,(MAX(D38:I38))-(MIN(D38:I38)))*7+1,0))),1))&amp;IF(H38=""," ",MID("▁▂▃▄▅▆▇█",MAX(1,MIN(8,ROUND((H38-(MIN(D38:I38)))/MAX(1E-9,(MAX(D38:I38))-(MIN(D38:I38)))*7+1,0))),1))&amp;IF(I38=""," ",MID("▁▂▃▄▅▆▇█",MAX(1,MIN(8,ROUND((I38-(MIN(D38:I38)))/MAX(1E-9,(MAX(D38:I38))-(MIN(D38:I38)))*7+1,0))),1))</f>
+        <v/>
+      </c>
       <c r="K38" s="2" t="n"/>
       <c r="L38" s="2" t="n"/>
+      <c r="N38" s="27" t="inlineStr">
+        <is>
+          <t>Renda</t>
+        </is>
+      </c>
+      <c r="O38" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="P38" s="28">
+        <f>IF(S38&gt;=0,S38,0)</f>
+        <v/>
+      </c>
+      <c r="Q38" s="28">
+        <f>IF(S38&lt;0,-S38,0)</f>
+        <v/>
+      </c>
+      <c r="R38" s="28">
+        <f>S38</f>
+        <v/>
+      </c>
+      <c r="S38" s="29">
+        <f>$Z$40</f>
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n"/>
-      <c r="B39" s="2" t="n"/>
-      <c r="C39" s="2" t="n"/>
-      <c r="D39" s="2" t="n"/>
-      <c r="E39" s="2" t="n"/>
-      <c r="F39" s="2" t="n"/>
-      <c r="G39" s="2" t="n"/>
-      <c r="H39" s="2" t="n"/>
-      <c r="I39" s="2" t="n"/>
-      <c r="J39" s="2" t="n"/>
+      <c r="B39" s="18" t="inlineStr">
+        <is>
+          <t>Score</t>
+        </is>
+      </c>
+      <c r="C39" s="24">
+        <f>$Z$47</f>
+        <v/>
+      </c>
+      <c r="D39" s="25" t="n">
+        <v>55</v>
+      </c>
+      <c r="E39" s="25" t="n">
+        <v>62</v>
+      </c>
+      <c r="F39" s="25" t="n">
+        <v>68</v>
+      </c>
+      <c r="G39" s="25" t="n">
+        <v>74</v>
+      </c>
+      <c r="H39" s="25" t="n">
+        <v>85</v>
+      </c>
+      <c r="I39" s="25">
+        <f>$Z$47</f>
+        <v/>
+      </c>
+      <c r="J39" s="26">
+        <f>IF(D39=""," ",MID("▁▂▃▄▅▆▇█",MAX(1,MIN(8,ROUND((D39-(MIN(D39:I39)))/MAX(1E-9,(MAX(D39:I39))-(MIN(D39:I39)))*7+1,0))),1))&amp;IF(E39=""," ",MID("▁▂▃▄▅▆▇█",MAX(1,MIN(8,ROUND((E39-(MIN(D39:I39)))/MAX(1E-9,(MAX(D39:I39))-(MIN(D39:I39)))*7+1,0))),1))&amp;IF(F39=""," ",MID("▁▂▃▄▅▆▇█",MAX(1,MIN(8,ROUND((F39-(MIN(D39:I39)))/MAX(1E-9,(MAX(D39:I39))-(MIN(D39:I39)))*7+1,0))),1))&amp;IF(G39=""," ",MID("▁▂▃▄▅▆▇█",MAX(1,MIN(8,ROUND((G39-(MIN(D39:I39)))/MAX(1E-9,(MAX(D39:I39))-(MIN(D39:I39)))*7+1,0))),1))&amp;IF(H39=""," ",MID("▁▂▃▄▅▆▇█",MAX(1,MIN(8,ROUND((H39-(MIN(D39:I39)))/MAX(1E-9,(MAX(D39:I39))-(MIN(D39:I39)))*7+1,0))),1))&amp;IF(I39=""," ",MID("▁▂▃▄▅▆▇█",MAX(1,MIN(8,ROUND((I39-(MIN(D39:I39)))/MAX(1E-9,(MAX(D39:I39))-(MIN(D39:I39)))*7+1,0))),1))</f>
+        <v/>
+      </c>
       <c r="K39" s="2" t="n"/>
       <c r="L39" s="2" t="n"/>
+      <c r="N39" s="27" t="inlineStr">
+        <is>
+          <t>Gastos</t>
+        </is>
+      </c>
+      <c r="O39" s="28">
+        <f>IF(S39&gt;=0,R38,R38+S39)</f>
+        <v/>
+      </c>
+      <c r="P39" s="28">
+        <f>IF(S39&gt;=0,S39,0)</f>
+        <v/>
+      </c>
+      <c r="Q39" s="28">
+        <f>IF(S39&lt;0,-S39,0)</f>
+        <v/>
+      </c>
+      <c r="R39" s="28">
+        <f>R38+S39</f>
+        <v/>
+      </c>
+      <c r="S39" s="29">
+        <f>-$Z$41</f>
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n"/>
-      <c r="B40" s="23">
-        <f>SUMIF(LANCAMENTOS!D:D,"Entrada",LANCAMENTOS!E:E)</f>
-        <v/>
-      </c>
-      <c r="C40" s="2" t="n"/>
-      <c r="D40" s="2" t="n"/>
-      <c r="E40" s="2" t="n"/>
-      <c r="F40" s="2" t="n"/>
-      <c r="G40" s="2" t="n"/>
-      <c r="H40" s="2" t="n"/>
-      <c r="I40" s="2" t="n"/>
-      <c r="J40" s="2" t="n"/>
+      <c r="B40" s="18" t="inlineStr">
+        <is>
+          <t>Investimentos</t>
+        </is>
+      </c>
+      <c r="C40" s="24">
+        <f>$Z$44</f>
+        <v/>
+      </c>
+      <c r="D40" s="25" t="n">
+        <v>400</v>
+      </c>
+      <c r="E40" s="25" t="n">
+        <v>600</v>
+      </c>
+      <c r="F40" s="25" t="n">
+        <v>800</v>
+      </c>
+      <c r="G40" s="25" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H40" s="25" t="n">
+        <v>1200</v>
+      </c>
+      <c r="I40" s="25">
+        <f>$Z$44</f>
+        <v/>
+      </c>
+      <c r="J40" s="26">
+        <f>IF(D40=""," ",MID("▁▂▃▄▅▆▇█",MAX(1,MIN(8,ROUND((D40-(MIN(D40:I40)))/MAX(1E-9,(MAX(D40:I40))-(MIN(D40:I40)))*7+1,0))),1))&amp;IF(E40=""," ",MID("▁▂▃▄▅▆▇█",MAX(1,MIN(8,ROUND((E40-(MIN(D40:I40)))/MAX(1E-9,(MAX(D40:I40))-(MIN(D40:I40)))*7+1,0))),1))&amp;IF(F40=""," ",MID("▁▂▃▄▅▆▇█",MAX(1,MIN(8,ROUND((F40-(MIN(D40:I40)))/MAX(1E-9,(MAX(D40:I40))-(MIN(D40:I40)))*7+1,0))),1))&amp;IF(G40=""," ",MID("▁▂▃▄▅▆▇█",MAX(1,MIN(8,ROUND((G40-(MIN(D40:I40)))/MAX(1E-9,(MAX(D40:I40))-(MIN(D40:I40)))*7+1,0))),1))&amp;IF(H40=""," ",MID("▁▂▃▄▅▆▇█",MAX(1,MIN(8,ROUND((H40-(MIN(D40:I40)))/MAX(1E-9,(MAX(D40:I40))-(MIN(D40:I40)))*7+1,0))),1))&amp;IF(I40=""," ",MID("▁▂▃▄▅▆▇█",MAX(1,MIN(8,ROUND((I40-(MIN(D40:I40)))/MAX(1E-9,(MAX(D40:I40))-(MIN(D40:I40)))*7+1,0))),1))</f>
+        <v/>
+      </c>
       <c r="K40" s="2" t="n"/>
       <c r="L40" s="2" t="n"/>
+      <c r="N40" s="27" t="inlineStr">
+        <is>
+          <t>Saldo</t>
+        </is>
+      </c>
+      <c r="O40" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="P40" s="28">
+        <f>IF(S40&gt;=0,S40,0)</f>
+        <v/>
+      </c>
+      <c r="Q40" s="28">
+        <f>IF(S40&lt;0,-S40,0)</f>
+        <v/>
+      </c>
+      <c r="R40" s="28">
+        <f>S40</f>
+        <v/>
+      </c>
+      <c r="S40" s="29">
+        <f>$Z$42</f>
+        <v/>
+      </c>
+      <c r="Z40" s="30">
+        <f>SUMIF(LANCAMENTOS!D:D,"Entrada",LANCAMENTOS!E:E)</f>
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n"/>
-      <c r="B41" s="23">
-        <f>SUMIF(LANCAMENTOS!D:D,"Saída",LANCAMENTOS!E:E)</f>
-        <v/>
-      </c>
-      <c r="C41" s="2" t="n"/>
-      <c r="D41" s="2" t="n"/>
-      <c r="E41" s="2" t="n"/>
-      <c r="F41" s="2" t="n"/>
-      <c r="G41" s="2" t="n"/>
-      <c r="H41" s="2" t="n"/>
-      <c r="I41" s="2" t="n"/>
-      <c r="J41" s="2" t="n"/>
+      <c r="B41" s="18" t="inlineStr">
+        <is>
+          <t>Dívidas</t>
+        </is>
+      </c>
+      <c r="C41" s="24">
+        <f>$Z$45</f>
+        <v/>
+      </c>
+      <c r="D41" s="25" t="n">
+        <v>1400</v>
+      </c>
+      <c r="E41" s="25" t="n">
+        <v>1200</v>
+      </c>
+      <c r="F41" s="25" t="n">
+        <v>1100</v>
+      </c>
+      <c r="G41" s="25" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H41" s="25" t="n">
+        <v>950</v>
+      </c>
+      <c r="I41" s="25">
+        <f>$Z$45</f>
+        <v/>
+      </c>
+      <c r="J41" s="26">
+        <f>IF(D41=""," ",MID("▁▂▃▄▅▆▇█",MAX(1,MIN(8,ROUND((D41-(MIN(D41:I41)))/MAX(1E-9,(MAX(D41:I41))-(MIN(D41:I41)))*7+1,0))),1))&amp;IF(E41=""," ",MID("▁▂▃▄▅▆▇█",MAX(1,MIN(8,ROUND((E41-(MIN(D41:I41)))/MAX(1E-9,(MAX(D41:I41))-(MIN(D41:I41)))*7+1,0))),1))&amp;IF(F41=""," ",MID("▁▂▃▄▅▆▇█",MAX(1,MIN(8,ROUND((F41-(MIN(D41:I41)))/MAX(1E-9,(MAX(D41:I41))-(MIN(D41:I41)))*7+1,0))),1))&amp;IF(G41=""," ",MID("▁▂▃▄▅▆▇█",MAX(1,MIN(8,ROUND((G41-(MIN(D41:I41)))/MAX(1E-9,(MAX(D41:I41))-(MIN(D41:I41)))*7+1,0))),1))&amp;IF(H41=""," ",MID("▁▂▃▄▅▆▇█",MAX(1,MIN(8,ROUND((H41-(MIN(D41:I41)))/MAX(1E-9,(MAX(D41:I41))-(MIN(D41:I41)))*7+1,0))),1))&amp;IF(I41=""," ",MID("▁▂▃▄▅▆▇█",MAX(1,MIN(8,ROUND((I41-(MIN(D41:I41)))/MAX(1E-9,(MAX(D41:I41))-(MIN(D41:I41)))*7+1,0))),1))</f>
+        <v/>
+      </c>
       <c r="K41" s="2" t="n"/>
       <c r="L41" s="2" t="n"/>
+      <c r="Z41" s="30">
+        <f>SUMIF(LANCAMENTOS!D:D,"Saída",LANCAMENTOS!E:E)</f>
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n"/>
-      <c r="B42" s="23">
-        <f>B40-B41</f>
-        <v/>
-      </c>
+      <c r="B42" s="2" t="n"/>
       <c r="C42" s="2" t="n"/>
       <c r="D42" s="2" t="n"/>
       <c r="E42" s="2" t="n"/>
@@ -1789,13 +2344,14 @@
       <c r="J42" s="2" t="n"/>
       <c r="K42" s="2" t="n"/>
       <c r="L42" s="2" t="n"/>
+      <c r="Z42" s="30">
+        <f>Z40-Z41</f>
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n"/>
-      <c r="B43" s="23">
-        <f>IFERROR(B42/B40,0)</f>
-        <v/>
-      </c>
+      <c r="B43" s="2" t="n"/>
       <c r="C43" s="2" t="n"/>
       <c r="D43" s="2" t="n"/>
       <c r="E43" s="2" t="n"/>
@@ -1806,13 +2362,14 @@
       <c r="J43" s="2" t="n"/>
       <c r="K43" s="2" t="n"/>
       <c r="L43" s="2" t="n"/>
+      <c r="Z43" s="30">
+        <f>IFERROR(Z42/Z40,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n"/>
-      <c r="B44" s="23">
-        <f>SUMIF(LANCAMENTOS!B:B,"Investimentos",LANCAMENTOS!E:E)</f>
-        <v/>
-      </c>
+      <c r="B44" s="2" t="n"/>
       <c r="C44" s="2" t="n"/>
       <c r="D44" s="2" t="n"/>
       <c r="E44" s="2" t="n"/>
@@ -1823,13 +2380,14 @@
       <c r="J44" s="2" t="n"/>
       <c r="K44" s="2" t="n"/>
       <c r="L44" s="2" t="n"/>
+      <c r="Z44" s="30">
+        <f>SUMIF(LANCAMENTOS!B:B,"Investimentos",LANCAMENTOS!E:E)</f>
+        <v/>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n"/>
-      <c r="B45" s="23">
-        <f>SUMIF(LANCAMENTOS!B:B,"Dívidas",LANCAMENTOS!E:E)</f>
-        <v/>
-      </c>
+      <c r="B45" s="2" t="n"/>
       <c r="C45" s="2" t="n"/>
       <c r="D45" s="2" t="n"/>
       <c r="E45" s="2" t="n"/>
@@ -1840,13 +2398,14 @@
       <c r="J45" s="2" t="n"/>
       <c r="K45" s="2" t="n"/>
       <c r="L45" s="2" t="n"/>
+      <c r="Z45" s="30">
+        <f>SUMIF(LANCAMENTOS!B:B,"Dívidas",LANCAMENTOS!E:E)</f>
+        <v/>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n"/>
-      <c r="B46" s="23">
-        <f>IFERROR(B41/B40,1)</f>
-        <v/>
-      </c>
+      <c r="B46" s="2" t="n"/>
       <c r="C46" s="2" t="n"/>
       <c r="D46" s="2" t="n"/>
       <c r="E46" s="2" t="n"/>
@@ -1857,13 +2416,14 @@
       <c r="J46" s="2" t="n"/>
       <c r="K46" s="2" t="n"/>
       <c r="L46" s="2" t="n"/>
+      <c r="Z46" s="30">
+        <f>IFERROR(Z41/Z40,1)</f>
+        <v/>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n"/>
-      <c r="B47" s="23">
-        <f>ROUND(MAX(0,MIN(100,MIN(40,MAX(0,B43)*160)+MIN(25,IFERROR(B44/B40,0)*250)+MAX(0,20-IFERROR(B45/B40,0)*100)+MAX(0,15-(B46-0.7)*50))),0)</f>
-        <v/>
-      </c>
+      <c r="B47" s="2" t="n"/>
       <c r="C47" s="2" t="n"/>
       <c r="D47" s="2" t="n"/>
       <c r="E47" s="2" t="n"/>
@@ -1874,6 +2434,10 @@
       <c r="J47" s="2" t="n"/>
       <c r="K47" s="2" t="n"/>
       <c r="L47" s="2" t="n"/>
+      <c r="Z47" s="30">
+        <f>ROUND(MAX(0,MIN(100,MIN(40,MAX(0,Z43)*160)+MIN(25,IFERROR(Z44/Z40,0)*250)+MAX(0,20-IFERROR(Z45/Z40,0)*100)+MAX(0,15-(Z46-0.7)*50))),0)</f>
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n"/>
@@ -1888,8 +2452,13 @@
       <c r="J48" s="2" t="n"/>
       <c r="K48" s="2" t="n"/>
       <c r="L48" s="2" t="n"/>
-    </row>
-    <row r="49">
+      <c r="N48" s="23" t="inlineStr">
+        <is>
+          <t>Spark · patrimônio 12m</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="26" customHeight="1">
       <c r="A49" s="2" t="n"/>
       <c r="B49" s="2" t="n"/>
       <c r="C49" s="2" t="n"/>
@@ -1902,6 +2471,21 @@
       <c r="J49" s="2" t="n"/>
       <c r="K49" s="2" t="n"/>
       <c r="L49" s="2" t="n"/>
+      <c r="N49" s="17" t="inlineStr">
+        <is>
+          <t>Ponto</t>
+        </is>
+      </c>
+      <c r="O49" s="17" t="inlineStr">
+        <is>
+          <t>Valor</t>
+        </is>
+      </c>
+      <c r="P49" s="31" t="inlineStr">
+        <is>
+          <t>Spark</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n"/>
@@ -1916,6 +2500,19 @@
       <c r="J50" s="2" t="n"/>
       <c r="K50" s="2" t="n"/>
       <c r="L50" s="2" t="n"/>
+      <c r="N50" s="32" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="O50" s="33">
+        <f>PROJECAO!B10</f>
+        <v/>
+      </c>
+      <c r="P50" s="34">
+        <f>IF(OR(O50="",NOT(ISNUMBER(O50))),"",REPT("▬",MAX(1,ROUND((O50-(MIN(O50:O61)))/MAX(1E-9,(MAX(O50:O61))-(MIN(O50:O61)))*10,0))))</f>
+        <v/>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n"/>
@@ -1930,6 +2527,19 @@
       <c r="J51" s="2" t="n"/>
       <c r="K51" s="2" t="n"/>
       <c r="L51" s="2" t="n"/>
+      <c r="N51" s="32" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="O51" s="33">
+        <f>PROJECAO!B11</f>
+        <v/>
+      </c>
+      <c r="P51" s="34">
+        <f>IF(OR(O51="",NOT(ISNUMBER(O51))),"",REPT("▬",MAX(1,ROUND((O51-(MIN(O50:O61)))/MAX(1E-9,(MAX(O50:O61))-(MIN(O50:O61)))*10,0))))</f>
+        <v/>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n"/>
@@ -1944,6 +2554,19 @@
       <c r="J52" s="2" t="n"/>
       <c r="K52" s="2" t="n"/>
       <c r="L52" s="2" t="n"/>
+      <c r="N52" s="32" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="O52" s="33">
+        <f>PROJECAO!B12</f>
+        <v/>
+      </c>
+      <c r="P52" s="34">
+        <f>IF(OR(O52="",NOT(ISNUMBER(O52))),"",REPT("▬",MAX(1,ROUND((O52-(MIN(O50:O61)))/MAX(1E-9,(MAX(O50:O61))-(MIN(O50:O61)))*10,0))))</f>
+        <v/>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n"/>
@@ -1958,6 +2581,19 @@
       <c r="J53" s="2" t="n"/>
       <c r="K53" s="2" t="n"/>
       <c r="L53" s="2" t="n"/>
+      <c r="N53" s="32" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="O53" s="33">
+        <f>PROJECAO!B13</f>
+        <v/>
+      </c>
+      <c r="P53" s="34">
+        <f>IF(OR(O53="",NOT(ISNUMBER(O53))),"",REPT("▬",MAX(1,ROUND((O53-(MIN(O50:O61)))/MAX(1E-9,(MAX(O50:O61))-(MIN(O50:O61)))*10,0))))</f>
+        <v/>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n"/>
@@ -1972,6 +2608,19 @@
       <c r="J54" s="2" t="n"/>
       <c r="K54" s="2" t="n"/>
       <c r="L54" s="2" t="n"/>
+      <c r="N54" s="32" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="O54" s="33">
+        <f>PROJECAO!B14</f>
+        <v/>
+      </c>
+      <c r="P54" s="34">
+        <f>IF(OR(O54="",NOT(ISNUMBER(O54))),"",REPT("▬",MAX(1,ROUND((O54-(MIN(O50:O61)))/MAX(1E-9,(MAX(O50:O61))-(MIN(O50:O61)))*10,0))))</f>
+        <v/>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n"/>
@@ -1986,6 +2635,19 @@
       <c r="J55" s="2" t="n"/>
       <c r="K55" s="2" t="n"/>
       <c r="L55" s="2" t="n"/>
+      <c r="N55" s="32" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="O55" s="33">
+        <f>PROJECAO!B15</f>
+        <v/>
+      </c>
+      <c r="P55" s="34">
+        <f>IF(OR(O55="",NOT(ISNUMBER(O55))),"",REPT("▬",MAX(1,ROUND((O55-(MIN(O50:O61)))/MAX(1E-9,(MAX(O50:O61))-(MIN(O50:O61)))*10,0))))</f>
+        <v/>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n"/>
@@ -2000,6 +2662,19 @@
       <c r="J56" s="2" t="n"/>
       <c r="K56" s="2" t="n"/>
       <c r="L56" s="2" t="n"/>
+      <c r="N56" s="32" t="inlineStr">
+        <is>
+          <t>M7</t>
+        </is>
+      </c>
+      <c r="O56" s="33">
+        <f>PROJECAO!B16</f>
+        <v/>
+      </c>
+      <c r="P56" s="34">
+        <f>IF(OR(O56="",NOT(ISNUMBER(O56))),"",REPT("▬",MAX(1,ROUND((O56-(MIN(O50:O61)))/MAX(1E-9,(MAX(O50:O61))-(MIN(O50:O61)))*10,0))))</f>
+        <v/>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n"/>
@@ -2014,6 +2689,19 @@
       <c r="J57" s="2" t="n"/>
       <c r="K57" s="2" t="n"/>
       <c r="L57" s="2" t="n"/>
+      <c r="N57" s="32" t="inlineStr">
+        <is>
+          <t>M8</t>
+        </is>
+      </c>
+      <c r="O57" s="33">
+        <f>PROJECAO!B17</f>
+        <v/>
+      </c>
+      <c r="P57" s="34">
+        <f>IF(OR(O57="",NOT(ISNUMBER(O57))),"",REPT("▬",MAX(1,ROUND((O57-(MIN(O50:O61)))/MAX(1E-9,(MAX(O50:O61))-(MIN(O50:O61)))*10,0))))</f>
+        <v/>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n"/>
@@ -2028,6 +2716,19 @@
       <c r="J58" s="2" t="n"/>
       <c r="K58" s="2" t="n"/>
       <c r="L58" s="2" t="n"/>
+      <c r="N58" s="32" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="O58" s="33">
+        <f>PROJECAO!B18</f>
+        <v/>
+      </c>
+      <c r="P58" s="34">
+        <f>IF(OR(O58="",NOT(ISNUMBER(O58))),"",REPT("▬",MAX(1,ROUND((O58-(MIN(O50:O61)))/MAX(1E-9,(MAX(O50:O61))-(MIN(O50:O61)))*10,0))))</f>
+        <v/>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n"/>
@@ -2042,6 +2743,19 @@
       <c r="J59" s="2" t="n"/>
       <c r="K59" s="2" t="n"/>
       <c r="L59" s="2" t="n"/>
+      <c r="N59" s="32" t="inlineStr">
+        <is>
+          <t>M10</t>
+        </is>
+      </c>
+      <c r="O59" s="33">
+        <f>PROJECAO!B19</f>
+        <v/>
+      </c>
+      <c r="P59" s="34">
+        <f>IF(OR(O59="",NOT(ISNUMBER(O59))),"",REPT("▬",MAX(1,ROUND((O59-(MIN(O50:O61)))/MAX(1E-9,(MAX(O50:O61))-(MIN(O50:O61)))*10,0))))</f>
+        <v/>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n"/>
@@ -2056,6 +2770,34 @@
       <c r="J60" s="2" t="n"/>
       <c r="K60" s="2" t="n"/>
       <c r="L60" s="2" t="n"/>
+      <c r="N60" s="32" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="O60" s="33">
+        <f>PROJECAO!B20</f>
+        <v/>
+      </c>
+      <c r="P60" s="34">
+        <f>IF(OR(O60="",NOT(ISNUMBER(O60))),"",REPT("▬",MAX(1,ROUND((O60-(MIN(O50:O61)))/MAX(1E-9,(MAX(O50:O61))-(MIN(O50:O61)))*10,0))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="N61" s="32" t="inlineStr">
+        <is>
+          <t>M12</t>
+        </is>
+      </c>
+      <c r="O61" s="33">
+        <f>PROJECAO!B21</f>
+        <v/>
+      </c>
+      <c r="P61" s="34">
+        <f>IF(OR(O61="",NOT(ISNUMBER(O61))),"",REPT("▬",MAX(1,ROUND((O61-(MIN(O50:O61)))/MAX(1E-9,(MAX(O50:O61))-(MIN(O50:O61)))*10,0))))</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="19">
@@ -2088,6 +2830,23 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="S38:S40">
+    <cfRule type="cellIs" priority="2" operator="greaterThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="lessThan" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C38:C41">
+    <cfRule type="dataBar" priority="4">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="00C99C66"/>
+      </dataBar>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -2149,7 +2908,7 @@
           <t>Tipo</t>
         </is>
       </c>
-      <c r="D3" s="24" t="inlineStr">
+      <c r="D3" s="35" t="inlineStr">
         <is>
           <t>Tipos de lançamento</t>
         </is>
@@ -2160,20 +2919,20 @@
       <c r="H3" s="2" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="25" t="inlineStr">
+      <c r="A4" s="36" t="inlineStr">
         <is>
           <t>Moradia</t>
         </is>
       </c>
-      <c r="B4" s="26" t="n">
+      <c r="B4" s="37" t="n">
         <v>0.3</v>
       </c>
-      <c r="C4" s="27" t="inlineStr">
+      <c r="C4" s="38" t="inlineStr">
         <is>
           <t>Essencial</t>
         </is>
       </c>
-      <c r="D4" s="25" t="inlineStr">
+      <c r="D4" s="36" t="inlineStr">
         <is>
           <t>Entrada</t>
         </is>
@@ -2184,20 +2943,20 @@
       <c r="H4" s="2" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="25" t="inlineStr">
+      <c r="A5" s="36" t="inlineStr">
         <is>
           <t>Alimentação</t>
         </is>
       </c>
-      <c r="B5" s="26" t="n">
+      <c r="B5" s="37" t="n">
         <v>0.15</v>
       </c>
-      <c r="C5" s="27" t="inlineStr">
+      <c r="C5" s="38" t="inlineStr">
         <is>
           <t>Essencial</t>
         </is>
       </c>
-      <c r="D5" s="25" t="inlineStr">
+      <c r="D5" s="36" t="inlineStr">
         <is>
           <t>Saída</t>
         </is>
@@ -2208,15 +2967,15 @@
       <c r="H5" s="2" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="25" t="inlineStr">
+      <c r="A6" s="36" t="inlineStr">
         <is>
           <t>Transporte</t>
         </is>
       </c>
-      <c r="B6" s="26" t="n">
+      <c r="B6" s="37" t="n">
         <v>0.1</v>
       </c>
-      <c r="C6" s="27" t="inlineStr">
+      <c r="C6" s="38" t="inlineStr">
         <is>
           <t>Essencial</t>
         </is>
@@ -2228,15 +2987,15 @@
       <c r="H6" s="2" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="25" t="inlineStr">
+      <c r="A7" s="36" t="inlineStr">
         <is>
           <t>Saúde</t>
         </is>
       </c>
-      <c r="B7" s="26" t="n">
+      <c r="B7" s="37" t="n">
         <v>0.08</v>
       </c>
-      <c r="C7" s="27" t="inlineStr">
+      <c r="C7" s="38" t="inlineStr">
         <is>
           <t>Essencial</t>
         </is>
@@ -2248,15 +3007,15 @@
       <c r="H7" s="2" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="25" t="inlineStr">
+      <c r="A8" s="36" t="inlineStr">
         <is>
           <t>Educação</t>
         </is>
       </c>
-      <c r="B8" s="26" t="n">
+      <c r="B8" s="37" t="n">
         <v>0.08</v>
       </c>
-      <c r="C8" s="27" t="inlineStr">
+      <c r="C8" s="38" t="inlineStr">
         <is>
           <t>Investimento</t>
         </is>
@@ -2268,15 +3027,15 @@
       <c r="H8" s="2" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="25" t="inlineStr">
+      <c r="A9" s="36" t="inlineStr">
         <is>
           <t>Lazer</t>
         </is>
       </c>
-      <c r="B9" s="26" t="n">
+      <c r="B9" s="37" t="n">
         <v>0.08</v>
       </c>
-      <c r="C9" s="27" t="inlineStr">
+      <c r="C9" s="38" t="inlineStr">
         <is>
           <t>Estilo de vida</t>
         </is>
@@ -2288,15 +3047,15 @@
       <c r="H9" s="2" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="25" t="inlineStr">
+      <c r="A10" s="36" t="inlineStr">
         <is>
           <t>Assinaturas</t>
         </is>
       </c>
-      <c r="B10" s="26" t="n">
+      <c r="B10" s="37" t="n">
         <v>0.05</v>
       </c>
-      <c r="C10" s="27" t="inlineStr">
+      <c r="C10" s="38" t="inlineStr">
         <is>
           <t>Estilo de vida</t>
         </is>
@@ -2308,15 +3067,15 @@
       <c r="H10" s="2" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="25" t="inlineStr">
+      <c r="A11" s="36" t="inlineStr">
         <is>
           <t>Investimentos</t>
         </is>
       </c>
-      <c r="B11" s="26" t="n">
+      <c r="B11" s="37" t="n">
         <v>0.15</v>
       </c>
-      <c r="C11" s="27" t="inlineStr">
+      <c r="C11" s="38" t="inlineStr">
         <is>
           <t>Futuro</t>
         </is>
@@ -2328,15 +3087,15 @@
       <c r="H11" s="2" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="25" t="inlineStr">
+      <c r="A12" s="36" t="inlineStr">
         <is>
           <t>Dívidas</t>
         </is>
       </c>
-      <c r="B12" s="26" t="n">
+      <c r="B12" s="37" t="n">
         <v>0.1</v>
       </c>
-      <c r="C12" s="27" t="inlineStr">
+      <c r="C12" s="38" t="inlineStr">
         <is>
           <t>Risco</t>
         </is>
@@ -2348,15 +3107,15 @@
       <c r="H12" s="2" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="25" t="inlineStr">
+      <c r="A13" s="36" t="inlineStr">
         <is>
           <t>Outros</t>
         </is>
       </c>
-      <c r="B13" s="26" t="n">
+      <c r="B13" s="37" t="n">
         <v>0.05</v>
       </c>
-      <c r="C13" s="27" t="inlineStr">
+      <c r="C13" s="38" t="inlineStr">
         <is>
           <t>Estilo de vida</t>
         </is>
@@ -2746,28 +3505,28 @@
       <c r="H5" s="2" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="28" t="n">
+      <c r="A6" s="39" t="n">
         <v>46205</v>
       </c>
-      <c r="B6" s="29" t="inlineStr">
+      <c r="B6" s="40" t="inlineStr">
         <is>
           <t>Entrada</t>
         </is>
       </c>
-      <c r="C6" s="29" t="inlineStr">
+      <c r="C6" s="40" t="inlineStr">
         <is>
           <t>Salário</t>
         </is>
       </c>
-      <c r="D6" s="29" t="inlineStr">
+      <c r="D6" s="40" t="inlineStr">
         <is>
           <t>Entrada</t>
         </is>
       </c>
-      <c r="E6" s="30" t="n">
+      <c r="E6" s="41" t="n">
         <v>9200</v>
       </c>
-      <c r="F6" s="29">
+      <c r="F6" s="40">
         <f>IF(D6&lt;&gt;"Saída","",IF(E6&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B6,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -2775,28 +3534,28 @@
       <c r="H6" s="2" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="28" t="n">
+      <c r="A7" s="39" t="n">
         <v>46206</v>
       </c>
-      <c r="B7" s="29" t="inlineStr">
+      <c r="B7" s="40" t="inlineStr">
         <is>
           <t>Moradia</t>
         </is>
       </c>
-      <c r="C7" s="29" t="inlineStr">
+      <c r="C7" s="40" t="inlineStr">
         <is>
           <t>Aluguel + condomínio</t>
         </is>
       </c>
-      <c r="D7" s="29" t="inlineStr">
+      <c r="D7" s="40" t="inlineStr">
         <is>
           <t>Saída</t>
         </is>
       </c>
-      <c r="E7" s="30" t="n">
+      <c r="E7" s="41" t="n">
         <v>2450</v>
       </c>
-      <c r="F7" s="29">
+      <c r="F7" s="40">
         <f>IF(D7&lt;&gt;"Saída","",IF(E7&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B7,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -2804,28 +3563,28 @@
       <c r="H7" s="2" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="28" t="n">
+      <c r="A8" s="39" t="n">
         <v>46207</v>
       </c>
-      <c r="B8" s="29" t="inlineStr">
+      <c r="B8" s="40" t="inlineStr">
         <is>
           <t>Alimentação</t>
         </is>
       </c>
-      <c r="C8" s="29" t="inlineStr">
+      <c r="C8" s="40" t="inlineStr">
         <is>
           <t>Mercado do mês</t>
         </is>
       </c>
-      <c r="D8" s="29" t="inlineStr">
+      <c r="D8" s="40" t="inlineStr">
         <is>
           <t>Saída</t>
         </is>
       </c>
-      <c r="E8" s="30" t="n">
+      <c r="E8" s="41" t="n">
         <v>1180</v>
       </c>
-      <c r="F8" s="29">
+      <c r="F8" s="40">
         <f>IF(D8&lt;&gt;"Saída","",IF(E8&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B8,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -2833,28 +3592,28 @@
       <c r="H8" s="2" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="28" t="n">
+      <c r="A9" s="39" t="n">
         <v>46208</v>
       </c>
-      <c r="B9" s="29" t="inlineStr">
+      <c r="B9" s="40" t="inlineStr">
         <is>
           <t>Assinaturas</t>
         </is>
       </c>
-      <c r="C9" s="29" t="inlineStr">
+      <c r="C9" s="40" t="inlineStr">
         <is>
           <t>Softwares e streaming</t>
         </is>
       </c>
-      <c r="D9" s="29" t="inlineStr">
+      <c r="D9" s="40" t="inlineStr">
         <is>
           <t>Saída</t>
         </is>
       </c>
-      <c r="E9" s="30" t="n">
+      <c r="E9" s="41" t="n">
         <v>320</v>
       </c>
-      <c r="F9" s="29">
+      <c r="F9" s="40">
         <f>IF(D9&lt;&gt;"Saída","",IF(E9&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B9,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -2862,28 +3621,28 @@
       <c r="H9" s="2" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="28" t="n">
+      <c r="A10" s="39" t="n">
         <v>46209</v>
       </c>
-      <c r="B10" s="29" t="inlineStr">
+      <c r="B10" s="40" t="inlineStr">
         <is>
           <t>Transporte</t>
         </is>
       </c>
-      <c r="C10" s="29" t="inlineStr">
+      <c r="C10" s="40" t="inlineStr">
         <is>
           <t>Combustível + app</t>
         </is>
       </c>
-      <c r="D10" s="29" t="inlineStr">
+      <c r="D10" s="40" t="inlineStr">
         <is>
           <t>Saída</t>
         </is>
       </c>
-      <c r="E10" s="30" t="n">
+      <c r="E10" s="41" t="n">
         <v>560</v>
       </c>
-      <c r="F10" s="29">
+      <c r="F10" s="40">
         <f>IF(D10&lt;&gt;"Saída","",IF(E10&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B10,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -2891,28 +3650,28 @@
       <c r="H10" s="2" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="28" t="n">
+      <c r="A11" s="39" t="n">
         <v>46210</v>
       </c>
-      <c r="B11" s="29" t="inlineStr">
+      <c r="B11" s="40" t="inlineStr">
         <is>
           <t>Entrada</t>
         </is>
       </c>
-      <c r="C11" s="29" t="inlineStr">
+      <c r="C11" s="40" t="inlineStr">
         <is>
           <t>Freelance</t>
         </is>
       </c>
-      <c r="D11" s="29" t="inlineStr">
+      <c r="D11" s="40" t="inlineStr">
         <is>
           <t>Entrada</t>
         </is>
       </c>
-      <c r="E11" s="30" t="n">
+      <c r="E11" s="41" t="n">
         <v>2400</v>
       </c>
-      <c r="F11" s="29">
+      <c r="F11" s="40">
         <f>IF(D11&lt;&gt;"Saída","",IF(E11&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B11,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -2920,28 +3679,28 @@
       <c r="H11" s="2" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="28" t="n">
+      <c r="A12" s="39" t="n">
         <v>46211</v>
       </c>
-      <c r="B12" s="29" t="inlineStr">
+      <c r="B12" s="40" t="inlineStr">
         <is>
           <t>Lazer</t>
         </is>
       </c>
-      <c r="C12" s="29" t="inlineStr">
+      <c r="C12" s="40" t="inlineStr">
         <is>
           <t>Restaurantes</t>
         </is>
       </c>
-      <c r="D12" s="29" t="inlineStr">
+      <c r="D12" s="40" t="inlineStr">
         <is>
           <t>Saída</t>
         </is>
       </c>
-      <c r="E12" s="30" t="n">
+      <c r="E12" s="41" t="n">
         <v>680</v>
       </c>
-      <c r="F12" s="29">
+      <c r="F12" s="40">
         <f>IF(D12&lt;&gt;"Saída","",IF(E12&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B12,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -2949,28 +3708,28 @@
       <c r="H12" s="2" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="28" t="n">
+      <c r="A13" s="39" t="n">
         <v>46212</v>
       </c>
-      <c r="B13" s="29" t="inlineStr">
+      <c r="B13" s="40" t="inlineStr">
         <is>
           <t>Saúde</t>
         </is>
       </c>
-      <c r="C13" s="29" t="inlineStr">
+      <c r="C13" s="40" t="inlineStr">
         <is>
           <t>Plano + farmácia</t>
         </is>
       </c>
-      <c r="D13" s="29" t="inlineStr">
+      <c r="D13" s="40" t="inlineStr">
         <is>
           <t>Saída</t>
         </is>
       </c>
-      <c r="E13" s="30" t="n">
+      <c r="E13" s="41" t="n">
         <v>540</v>
       </c>
-      <c r="F13" s="29">
+      <c r="F13" s="40">
         <f>IF(D13&lt;&gt;"Saída","",IF(E13&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B13,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -2978,28 +3737,28 @@
       <c r="H13" s="2" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="28" t="n">
+      <c r="A14" s="39" t="n">
         <v>46214</v>
       </c>
-      <c r="B14" s="29" t="inlineStr">
+      <c r="B14" s="40" t="inlineStr">
         <is>
           <t>Investimentos</t>
         </is>
       </c>
-      <c r="C14" s="29" t="inlineStr">
+      <c r="C14" s="40" t="inlineStr">
         <is>
           <t>Aporte carteira</t>
         </is>
       </c>
-      <c r="D14" s="29" t="inlineStr">
+      <c r="D14" s="40" t="inlineStr">
         <is>
           <t>Saída</t>
         </is>
       </c>
-      <c r="E14" s="30" t="n">
+      <c r="E14" s="41" t="n">
         <v>1500</v>
       </c>
-      <c r="F14" s="29">
+      <c r="F14" s="40">
         <f>IF(D14&lt;&gt;"Saída","",IF(E14&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B14,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3007,28 +3766,28 @@
       <c r="H14" s="2" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="28" t="n">
+      <c r="A15" s="39" t="n">
         <v>46216</v>
       </c>
-      <c r="B15" s="29" t="inlineStr">
+      <c r="B15" s="40" t="inlineStr">
         <is>
           <t>Dívidas</t>
         </is>
       </c>
-      <c r="C15" s="29" t="inlineStr">
+      <c r="C15" s="40" t="inlineStr">
         <is>
           <t>Cartão parcelado</t>
         </is>
       </c>
-      <c r="D15" s="29" t="inlineStr">
+      <c r="D15" s="40" t="inlineStr">
         <is>
           <t>Saída</t>
         </is>
       </c>
-      <c r="E15" s="30" t="n">
+      <c r="E15" s="41" t="n">
         <v>900</v>
       </c>
-      <c r="F15" s="29">
+      <c r="F15" s="40">
         <f>IF(D15&lt;&gt;"Saída","",IF(E15&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B15,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3036,12 +3795,12 @@
       <c r="H15" s="2" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="28" t="n"/>
-      <c r="B16" s="29" t="n"/>
-      <c r="C16" s="29" t="n"/>
-      <c r="D16" s="29" t="n"/>
-      <c r="E16" s="30" t="n"/>
-      <c r="F16" s="29">
+      <c r="A16" s="39" t="n"/>
+      <c r="B16" s="40" t="n"/>
+      <c r="C16" s="40" t="n"/>
+      <c r="D16" s="40" t="n"/>
+      <c r="E16" s="41" t="n"/>
+      <c r="F16" s="40">
         <f>IF(D16&lt;&gt;"Saída","",IF(E16&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B16,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3049,12 +3808,12 @@
       <c r="H16" s="2" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="28" t="n"/>
-      <c r="B17" s="29" t="n"/>
-      <c r="C17" s="29" t="n"/>
-      <c r="D17" s="29" t="n"/>
-      <c r="E17" s="30" t="n"/>
-      <c r="F17" s="29">
+      <c r="A17" s="39" t="n"/>
+      <c r="B17" s="40" t="n"/>
+      <c r="C17" s="40" t="n"/>
+      <c r="D17" s="40" t="n"/>
+      <c r="E17" s="41" t="n"/>
+      <c r="F17" s="40">
         <f>IF(D17&lt;&gt;"Saída","",IF(E17&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B17,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3062,12 +3821,12 @@
       <c r="H17" s="2" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="28" t="n"/>
-      <c r="B18" s="29" t="n"/>
-      <c r="C18" s="29" t="n"/>
-      <c r="D18" s="29" t="n"/>
-      <c r="E18" s="30" t="n"/>
-      <c r="F18" s="29">
+      <c r="A18" s="39" t="n"/>
+      <c r="B18" s="40" t="n"/>
+      <c r="C18" s="40" t="n"/>
+      <c r="D18" s="40" t="n"/>
+      <c r="E18" s="41" t="n"/>
+      <c r="F18" s="40">
         <f>IF(D18&lt;&gt;"Saída","",IF(E18&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B18,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3075,12 +3834,12 @@
       <c r="H18" s="2" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="28" t="n"/>
-      <c r="B19" s="29" t="n"/>
-      <c r="C19" s="29" t="n"/>
-      <c r="D19" s="29" t="n"/>
-      <c r="E19" s="30" t="n"/>
-      <c r="F19" s="29">
+      <c r="A19" s="39" t="n"/>
+      <c r="B19" s="40" t="n"/>
+      <c r="C19" s="40" t="n"/>
+      <c r="D19" s="40" t="n"/>
+      <c r="E19" s="41" t="n"/>
+      <c r="F19" s="40">
         <f>IF(D19&lt;&gt;"Saída","",IF(E19&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B19,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3088,12 +3847,12 @@
       <c r="H19" s="2" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="28" t="n"/>
-      <c r="B20" s="29" t="n"/>
-      <c r="C20" s="29" t="n"/>
-      <c r="D20" s="29" t="n"/>
-      <c r="E20" s="30" t="n"/>
-      <c r="F20" s="29">
+      <c r="A20" s="39" t="n"/>
+      <c r="B20" s="40" t="n"/>
+      <c r="C20" s="40" t="n"/>
+      <c r="D20" s="40" t="n"/>
+      <c r="E20" s="41" t="n"/>
+      <c r="F20" s="40">
         <f>IF(D20&lt;&gt;"Saída","",IF(E20&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B20,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3101,12 +3860,12 @@
       <c r="H20" s="2" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="28" t="n"/>
-      <c r="B21" s="29" t="n"/>
-      <c r="C21" s="29" t="n"/>
-      <c r="D21" s="29" t="n"/>
-      <c r="E21" s="30" t="n"/>
-      <c r="F21" s="29">
+      <c r="A21" s="39" t="n"/>
+      <c r="B21" s="40" t="n"/>
+      <c r="C21" s="40" t="n"/>
+      <c r="D21" s="40" t="n"/>
+      <c r="E21" s="41" t="n"/>
+      <c r="F21" s="40">
         <f>IF(D21&lt;&gt;"Saída","",IF(E21&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B21,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3114,12 +3873,12 @@
       <c r="H21" s="2" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="28" t="n"/>
-      <c r="B22" s="29" t="n"/>
-      <c r="C22" s="29" t="n"/>
-      <c r="D22" s="29" t="n"/>
-      <c r="E22" s="30" t="n"/>
-      <c r="F22" s="29">
+      <c r="A22" s="39" t="n"/>
+      <c r="B22" s="40" t="n"/>
+      <c r="C22" s="40" t="n"/>
+      <c r="D22" s="40" t="n"/>
+      <c r="E22" s="41" t="n"/>
+      <c r="F22" s="40">
         <f>IF(D22&lt;&gt;"Saída","",IF(E22&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B22,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3127,12 +3886,12 @@
       <c r="H22" s="2" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="28" t="n"/>
-      <c r="B23" s="29" t="n"/>
-      <c r="C23" s="29" t="n"/>
-      <c r="D23" s="29" t="n"/>
-      <c r="E23" s="30" t="n"/>
-      <c r="F23" s="29">
+      <c r="A23" s="39" t="n"/>
+      <c r="B23" s="40" t="n"/>
+      <c r="C23" s="40" t="n"/>
+      <c r="D23" s="40" t="n"/>
+      <c r="E23" s="41" t="n"/>
+      <c r="F23" s="40">
         <f>IF(D23&lt;&gt;"Saída","",IF(E23&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B23,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3140,12 +3899,12 @@
       <c r="H23" s="2" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="28" t="n"/>
-      <c r="B24" s="29" t="n"/>
-      <c r="C24" s="29" t="n"/>
-      <c r="D24" s="29" t="n"/>
-      <c r="E24" s="30" t="n"/>
-      <c r="F24" s="29">
+      <c r="A24" s="39" t="n"/>
+      <c r="B24" s="40" t="n"/>
+      <c r="C24" s="40" t="n"/>
+      <c r="D24" s="40" t="n"/>
+      <c r="E24" s="41" t="n"/>
+      <c r="F24" s="40">
         <f>IF(D24&lt;&gt;"Saída","",IF(E24&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B24,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3153,12 +3912,12 @@
       <c r="H24" s="2" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="28" t="n"/>
-      <c r="B25" s="29" t="n"/>
-      <c r="C25" s="29" t="n"/>
-      <c r="D25" s="29" t="n"/>
-      <c r="E25" s="30" t="n"/>
-      <c r="F25" s="29">
+      <c r="A25" s="39" t="n"/>
+      <c r="B25" s="40" t="n"/>
+      <c r="C25" s="40" t="n"/>
+      <c r="D25" s="40" t="n"/>
+      <c r="E25" s="41" t="n"/>
+      <c r="F25" s="40">
         <f>IF(D25&lt;&gt;"Saída","",IF(E25&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B25,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3166,12 +3925,12 @@
       <c r="H25" s="2" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="28" t="n"/>
-      <c r="B26" s="29" t="n"/>
-      <c r="C26" s="29" t="n"/>
-      <c r="D26" s="29" t="n"/>
-      <c r="E26" s="30" t="n"/>
-      <c r="F26" s="29">
+      <c r="A26" s="39" t="n"/>
+      <c r="B26" s="40" t="n"/>
+      <c r="C26" s="40" t="n"/>
+      <c r="D26" s="40" t="n"/>
+      <c r="E26" s="41" t="n"/>
+      <c r="F26" s="40">
         <f>IF(D26&lt;&gt;"Saída","",IF(E26&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B26,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3179,12 +3938,12 @@
       <c r="H26" s="2" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="28" t="n"/>
-      <c r="B27" s="29" t="n"/>
-      <c r="C27" s="29" t="n"/>
-      <c r="D27" s="29" t="n"/>
-      <c r="E27" s="30" t="n"/>
-      <c r="F27" s="29">
+      <c r="A27" s="39" t="n"/>
+      <c r="B27" s="40" t="n"/>
+      <c r="C27" s="40" t="n"/>
+      <c r="D27" s="40" t="n"/>
+      <c r="E27" s="41" t="n"/>
+      <c r="F27" s="40">
         <f>IF(D27&lt;&gt;"Saída","",IF(E27&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B27,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3192,12 +3951,12 @@
       <c r="H27" s="2" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="28" t="n"/>
-      <c r="B28" s="29" t="n"/>
-      <c r="C28" s="29" t="n"/>
-      <c r="D28" s="29" t="n"/>
-      <c r="E28" s="30" t="n"/>
-      <c r="F28" s="29">
+      <c r="A28" s="39" t="n"/>
+      <c r="B28" s="40" t="n"/>
+      <c r="C28" s="40" t="n"/>
+      <c r="D28" s="40" t="n"/>
+      <c r="E28" s="41" t="n"/>
+      <c r="F28" s="40">
         <f>IF(D28&lt;&gt;"Saída","",IF(E28&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B28,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3205,12 +3964,12 @@
       <c r="H28" s="2" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="28" t="n"/>
-      <c r="B29" s="29" t="n"/>
-      <c r="C29" s="29" t="n"/>
-      <c r="D29" s="29" t="n"/>
-      <c r="E29" s="30" t="n"/>
-      <c r="F29" s="29">
+      <c r="A29" s="39" t="n"/>
+      <c r="B29" s="40" t="n"/>
+      <c r="C29" s="40" t="n"/>
+      <c r="D29" s="40" t="n"/>
+      <c r="E29" s="41" t="n"/>
+      <c r="F29" s="40">
         <f>IF(D29&lt;&gt;"Saída","",IF(E29&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B29,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3218,12 +3977,12 @@
       <c r="H29" s="2" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="28" t="n"/>
-      <c r="B30" s="29" t="n"/>
-      <c r="C30" s="29" t="n"/>
-      <c r="D30" s="29" t="n"/>
-      <c r="E30" s="30" t="n"/>
-      <c r="F30" s="29">
+      <c r="A30" s="39" t="n"/>
+      <c r="B30" s="40" t="n"/>
+      <c r="C30" s="40" t="n"/>
+      <c r="D30" s="40" t="n"/>
+      <c r="E30" s="41" t="n"/>
+      <c r="F30" s="40">
         <f>IF(D30&lt;&gt;"Saída","",IF(E30&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B30,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3231,12 +3990,12 @@
       <c r="H30" s="2" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="28" t="n"/>
-      <c r="B31" s="29" t="n"/>
-      <c r="C31" s="29" t="n"/>
-      <c r="D31" s="29" t="n"/>
-      <c r="E31" s="30" t="n"/>
-      <c r="F31" s="29">
+      <c r="A31" s="39" t="n"/>
+      <c r="B31" s="40" t="n"/>
+      <c r="C31" s="40" t="n"/>
+      <c r="D31" s="40" t="n"/>
+      <c r="E31" s="41" t="n"/>
+      <c r="F31" s="40">
         <f>IF(D31&lt;&gt;"Saída","",IF(E31&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B31,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3244,12 +4003,12 @@
       <c r="H31" s="2" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="28" t="n"/>
-      <c r="B32" s="29" t="n"/>
-      <c r="C32" s="29" t="n"/>
-      <c r="D32" s="29" t="n"/>
-      <c r="E32" s="30" t="n"/>
-      <c r="F32" s="29">
+      <c r="A32" s="39" t="n"/>
+      <c r="B32" s="40" t="n"/>
+      <c r="C32" s="40" t="n"/>
+      <c r="D32" s="40" t="n"/>
+      <c r="E32" s="41" t="n"/>
+      <c r="F32" s="40">
         <f>IF(D32&lt;&gt;"Saída","",IF(E32&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B32,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3257,12 +4016,12 @@
       <c r="H32" s="2" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="28" t="n"/>
-      <c r="B33" s="29" t="n"/>
-      <c r="C33" s="29" t="n"/>
-      <c r="D33" s="29" t="n"/>
-      <c r="E33" s="30" t="n"/>
-      <c r="F33" s="29">
+      <c r="A33" s="39" t="n"/>
+      <c r="B33" s="40" t="n"/>
+      <c r="C33" s="40" t="n"/>
+      <c r="D33" s="40" t="n"/>
+      <c r="E33" s="41" t="n"/>
+      <c r="F33" s="40">
         <f>IF(D33&lt;&gt;"Saída","",IF(E33&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B33,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3270,12 +4029,12 @@
       <c r="H33" s="2" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="28" t="n"/>
-      <c r="B34" s="29" t="n"/>
-      <c r="C34" s="29" t="n"/>
-      <c r="D34" s="29" t="n"/>
-      <c r="E34" s="30" t="n"/>
-      <c r="F34" s="29">
+      <c r="A34" s="39" t="n"/>
+      <c r="B34" s="40" t="n"/>
+      <c r="C34" s="40" t="n"/>
+      <c r="D34" s="40" t="n"/>
+      <c r="E34" s="41" t="n"/>
+      <c r="F34" s="40">
         <f>IF(D34&lt;&gt;"Saída","",IF(E34&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B34,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3283,12 +4042,12 @@
       <c r="H34" s="2" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="28" t="n"/>
-      <c r="B35" s="29" t="n"/>
-      <c r="C35" s="29" t="n"/>
-      <c r="D35" s="29" t="n"/>
-      <c r="E35" s="30" t="n"/>
-      <c r="F35" s="29">
+      <c r="A35" s="39" t="n"/>
+      <c r="B35" s="40" t="n"/>
+      <c r="C35" s="40" t="n"/>
+      <c r="D35" s="40" t="n"/>
+      <c r="E35" s="41" t="n"/>
+      <c r="F35" s="40">
         <f>IF(D35&lt;&gt;"Saída","",IF(E35&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B35,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3296,12 +4055,12 @@
       <c r="H35" s="2" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="28" t="n"/>
-      <c r="B36" s="29" t="n"/>
-      <c r="C36" s="29" t="n"/>
-      <c r="D36" s="29" t="n"/>
-      <c r="E36" s="30" t="n"/>
-      <c r="F36" s="29">
+      <c r="A36" s="39" t="n"/>
+      <c r="B36" s="40" t="n"/>
+      <c r="C36" s="40" t="n"/>
+      <c r="D36" s="40" t="n"/>
+      <c r="E36" s="41" t="n"/>
+      <c r="F36" s="40">
         <f>IF(D36&lt;&gt;"Saída","",IF(E36&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B36,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3309,12 +4068,12 @@
       <c r="H36" s="2" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="28" t="n"/>
-      <c r="B37" s="29" t="n"/>
-      <c r="C37" s="29" t="n"/>
-      <c r="D37" s="29" t="n"/>
-      <c r="E37" s="30" t="n"/>
-      <c r="F37" s="29">
+      <c r="A37" s="39" t="n"/>
+      <c r="B37" s="40" t="n"/>
+      <c r="C37" s="40" t="n"/>
+      <c r="D37" s="40" t="n"/>
+      <c r="E37" s="41" t="n"/>
+      <c r="F37" s="40">
         <f>IF(D37&lt;&gt;"Saída","",IF(E37&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B37,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3322,12 +4081,12 @@
       <c r="H37" s="2" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="28" t="n"/>
-      <c r="B38" s="29" t="n"/>
-      <c r="C38" s="29" t="n"/>
-      <c r="D38" s="29" t="n"/>
-      <c r="E38" s="30" t="n"/>
-      <c r="F38" s="29">
+      <c r="A38" s="39" t="n"/>
+      <c r="B38" s="40" t="n"/>
+      <c r="C38" s="40" t="n"/>
+      <c r="D38" s="40" t="n"/>
+      <c r="E38" s="41" t="n"/>
+      <c r="F38" s="40">
         <f>IF(D38&lt;&gt;"Saída","",IF(E38&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B38,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3335,12 +4094,12 @@
       <c r="H38" s="2" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="28" t="n"/>
-      <c r="B39" s="29" t="n"/>
-      <c r="C39" s="29" t="n"/>
-      <c r="D39" s="29" t="n"/>
-      <c r="E39" s="30" t="n"/>
-      <c r="F39" s="29">
+      <c r="A39" s="39" t="n"/>
+      <c r="B39" s="40" t="n"/>
+      <c r="C39" s="40" t="n"/>
+      <c r="D39" s="40" t="n"/>
+      <c r="E39" s="41" t="n"/>
+      <c r="F39" s="40">
         <f>IF(D39&lt;&gt;"Saída","",IF(E39&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B39,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3348,12 +4107,12 @@
       <c r="H39" s="2" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="28" t="n"/>
-      <c r="B40" s="29" t="n"/>
-      <c r="C40" s="29" t="n"/>
-      <c r="D40" s="29" t="n"/>
-      <c r="E40" s="30" t="n"/>
-      <c r="F40" s="29">
+      <c r="A40" s="39" t="n"/>
+      <c r="B40" s="40" t="n"/>
+      <c r="C40" s="40" t="n"/>
+      <c r="D40" s="40" t="n"/>
+      <c r="E40" s="41" t="n"/>
+      <c r="F40" s="40">
         <f>IF(D40&lt;&gt;"Saída","",IF(E40&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B40,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3361,12 +4120,12 @@
       <c r="H40" s="2" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="28" t="n"/>
-      <c r="B41" s="29" t="n"/>
-      <c r="C41" s="29" t="n"/>
-      <c r="D41" s="29" t="n"/>
-      <c r="E41" s="30" t="n"/>
-      <c r="F41" s="29">
+      <c r="A41" s="39" t="n"/>
+      <c r="B41" s="40" t="n"/>
+      <c r="C41" s="40" t="n"/>
+      <c r="D41" s="40" t="n"/>
+      <c r="E41" s="41" t="n"/>
+      <c r="F41" s="40">
         <f>IF(D41&lt;&gt;"Saída","",IF(E41&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B41,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3374,12 +4133,12 @@
       <c r="H41" s="2" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="28" t="n"/>
-      <c r="B42" s="29" t="n"/>
-      <c r="C42" s="29" t="n"/>
-      <c r="D42" s="29" t="n"/>
-      <c r="E42" s="30" t="n"/>
-      <c r="F42" s="29">
+      <c r="A42" s="39" t="n"/>
+      <c r="B42" s="40" t="n"/>
+      <c r="C42" s="40" t="n"/>
+      <c r="D42" s="40" t="n"/>
+      <c r="E42" s="41" t="n"/>
+      <c r="F42" s="40">
         <f>IF(D42&lt;&gt;"Saída","",IF(E42&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B42,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3387,12 +4146,12 @@
       <c r="H42" s="2" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="28" t="n"/>
-      <c r="B43" s="29" t="n"/>
-      <c r="C43" s="29" t="n"/>
-      <c r="D43" s="29" t="n"/>
-      <c r="E43" s="30" t="n"/>
-      <c r="F43" s="29">
+      <c r="A43" s="39" t="n"/>
+      <c r="B43" s="40" t="n"/>
+      <c r="C43" s="40" t="n"/>
+      <c r="D43" s="40" t="n"/>
+      <c r="E43" s="41" t="n"/>
+      <c r="F43" s="40">
         <f>IF(D43&lt;&gt;"Saída","",IF(E43&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B43,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3400,12 +4159,12 @@
       <c r="H43" s="2" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="28" t="n"/>
-      <c r="B44" s="29" t="n"/>
-      <c r="C44" s="29" t="n"/>
-      <c r="D44" s="29" t="n"/>
-      <c r="E44" s="30" t="n"/>
-      <c r="F44" s="29">
+      <c r="A44" s="39" t="n"/>
+      <c r="B44" s="40" t="n"/>
+      <c r="C44" s="40" t="n"/>
+      <c r="D44" s="40" t="n"/>
+      <c r="E44" s="41" t="n"/>
+      <c r="F44" s="40">
         <f>IF(D44&lt;&gt;"Saída","",IF(E44&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B44,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3413,12 +4172,12 @@
       <c r="H44" s="2" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="28" t="n"/>
-      <c r="B45" s="29" t="n"/>
-      <c r="C45" s="29" t="n"/>
-      <c r="D45" s="29" t="n"/>
-      <c r="E45" s="30" t="n"/>
-      <c r="F45" s="29">
+      <c r="A45" s="39" t="n"/>
+      <c r="B45" s="40" t="n"/>
+      <c r="C45" s="40" t="n"/>
+      <c r="D45" s="40" t="n"/>
+      <c r="E45" s="41" t="n"/>
+      <c r="F45" s="40">
         <f>IF(D45&lt;&gt;"Saída","",IF(E45&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B45,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3426,12 +4185,12 @@
       <c r="H45" s="2" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="28" t="n"/>
-      <c r="B46" s="29" t="n"/>
-      <c r="C46" s="29" t="n"/>
-      <c r="D46" s="29" t="n"/>
-      <c r="E46" s="30" t="n"/>
-      <c r="F46" s="29">
+      <c r="A46" s="39" t="n"/>
+      <c r="B46" s="40" t="n"/>
+      <c r="C46" s="40" t="n"/>
+      <c r="D46" s="40" t="n"/>
+      <c r="E46" s="41" t="n"/>
+      <c r="F46" s="40">
         <f>IF(D46&lt;&gt;"Saída","",IF(E46&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B46,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3439,12 +4198,12 @@
       <c r="H46" s="2" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="28" t="n"/>
-      <c r="B47" s="29" t="n"/>
-      <c r="C47" s="29" t="n"/>
-      <c r="D47" s="29" t="n"/>
-      <c r="E47" s="30" t="n"/>
-      <c r="F47" s="29">
+      <c r="A47" s="39" t="n"/>
+      <c r="B47" s="40" t="n"/>
+      <c r="C47" s="40" t="n"/>
+      <c r="D47" s="40" t="n"/>
+      <c r="E47" s="41" t="n"/>
+      <c r="F47" s="40">
         <f>IF(D47&lt;&gt;"Saída","",IF(E47&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B47,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3452,12 +4211,12 @@
       <c r="H47" s="2" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="28" t="n"/>
-      <c r="B48" s="29" t="n"/>
-      <c r="C48" s="29" t="n"/>
-      <c r="D48" s="29" t="n"/>
-      <c r="E48" s="30" t="n"/>
-      <c r="F48" s="29">
+      <c r="A48" s="39" t="n"/>
+      <c r="B48" s="40" t="n"/>
+      <c r="C48" s="40" t="n"/>
+      <c r="D48" s="40" t="n"/>
+      <c r="E48" s="41" t="n"/>
+      <c r="F48" s="40">
         <f>IF(D48&lt;&gt;"Saída","",IF(E48&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B48,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3465,12 +4224,12 @@
       <c r="H48" s="2" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="28" t="n"/>
-      <c r="B49" s="29" t="n"/>
-      <c r="C49" s="29" t="n"/>
-      <c r="D49" s="29" t="n"/>
-      <c r="E49" s="30" t="n"/>
-      <c r="F49" s="29">
+      <c r="A49" s="39" t="n"/>
+      <c r="B49" s="40" t="n"/>
+      <c r="C49" s="40" t="n"/>
+      <c r="D49" s="40" t="n"/>
+      <c r="E49" s="41" t="n"/>
+      <c r="F49" s="40">
         <f>IF(D49&lt;&gt;"Saída","",IF(E49&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B49,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3478,12 +4237,12 @@
       <c r="H49" s="2" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="28" t="n"/>
-      <c r="B50" s="29" t="n"/>
-      <c r="C50" s="29" t="n"/>
-      <c r="D50" s="29" t="n"/>
-      <c r="E50" s="30" t="n"/>
-      <c r="F50" s="29">
+      <c r="A50" s="39" t="n"/>
+      <c r="B50" s="40" t="n"/>
+      <c r="C50" s="40" t="n"/>
+      <c r="D50" s="40" t="n"/>
+      <c r="E50" s="41" t="n"/>
+      <c r="F50" s="40">
         <f>IF(D50&lt;&gt;"Saída","",IF(E50&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B50,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3491,12 +4250,12 @@
       <c r="H50" s="2" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="28" t="n"/>
-      <c r="B51" s="29" t="n"/>
-      <c r="C51" s="29" t="n"/>
-      <c r="D51" s="29" t="n"/>
-      <c r="E51" s="30" t="n"/>
-      <c r="F51" s="29">
+      <c r="A51" s="39" t="n"/>
+      <c r="B51" s="40" t="n"/>
+      <c r="C51" s="40" t="n"/>
+      <c r="D51" s="40" t="n"/>
+      <c r="E51" s="41" t="n"/>
+      <c r="F51" s="40">
         <f>IF(D51&lt;&gt;"Saída","",IF(E51&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B51,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3504,12 +4263,12 @@
       <c r="H51" s="2" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="28" t="n"/>
-      <c r="B52" s="29" t="n"/>
-      <c r="C52" s="29" t="n"/>
-      <c r="D52" s="29" t="n"/>
-      <c r="E52" s="30" t="n"/>
-      <c r="F52" s="29">
+      <c r="A52" s="39" t="n"/>
+      <c r="B52" s="40" t="n"/>
+      <c r="C52" s="40" t="n"/>
+      <c r="D52" s="40" t="n"/>
+      <c r="E52" s="41" t="n"/>
+      <c r="F52" s="40">
         <f>IF(D52&lt;&gt;"Saída","",IF(E52&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B52,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3517,12 +4276,12 @@
       <c r="H52" s="2" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="28" t="n"/>
-      <c r="B53" s="29" t="n"/>
-      <c r="C53" s="29" t="n"/>
-      <c r="D53" s="29" t="n"/>
-      <c r="E53" s="30" t="n"/>
-      <c r="F53" s="29">
+      <c r="A53" s="39" t="n"/>
+      <c r="B53" s="40" t="n"/>
+      <c r="C53" s="40" t="n"/>
+      <c r="D53" s="40" t="n"/>
+      <c r="E53" s="41" t="n"/>
+      <c r="F53" s="40">
         <f>IF(D53&lt;&gt;"Saída","",IF(E53&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B53,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3530,12 +4289,12 @@
       <c r="H53" s="2" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="28" t="n"/>
-      <c r="B54" s="29" t="n"/>
-      <c r="C54" s="29" t="n"/>
-      <c r="D54" s="29" t="n"/>
-      <c r="E54" s="30" t="n"/>
-      <c r="F54" s="29">
+      <c r="A54" s="39" t="n"/>
+      <c r="B54" s="40" t="n"/>
+      <c r="C54" s="40" t="n"/>
+      <c r="D54" s="40" t="n"/>
+      <c r="E54" s="41" t="n"/>
+      <c r="F54" s="40">
         <f>IF(D54&lt;&gt;"Saída","",IF(E54&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B54,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3543,12 +4302,12 @@
       <c r="H54" s="2" t="n"/>
     </row>
     <row r="55">
-      <c r="A55" s="28" t="n"/>
-      <c r="B55" s="29" t="n"/>
-      <c r="C55" s="29" t="n"/>
-      <c r="D55" s="29" t="n"/>
-      <c r="E55" s="30" t="n"/>
-      <c r="F55" s="29">
+      <c r="A55" s="39" t="n"/>
+      <c r="B55" s="40" t="n"/>
+      <c r="C55" s="40" t="n"/>
+      <c r="D55" s="40" t="n"/>
+      <c r="E55" s="41" t="n"/>
+      <c r="F55" s="40">
         <f>IF(D55&lt;&gt;"Saída","",IF(E55&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B55,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3556,12 +4315,12 @@
       <c r="H55" s="2" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" s="28" t="n"/>
-      <c r="B56" s="29" t="n"/>
-      <c r="C56" s="29" t="n"/>
-      <c r="D56" s="29" t="n"/>
-      <c r="E56" s="30" t="n"/>
-      <c r="F56" s="29">
+      <c r="A56" s="39" t="n"/>
+      <c r="B56" s="40" t="n"/>
+      <c r="C56" s="40" t="n"/>
+      <c r="D56" s="40" t="n"/>
+      <c r="E56" s="41" t="n"/>
+      <c r="F56" s="40">
         <f>IF(D56&lt;&gt;"Saída","",IF(E56&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B56,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3569,12 +4328,12 @@
       <c r="H56" s="2" t="n"/>
     </row>
     <row r="57">
-      <c r="A57" s="28" t="n"/>
-      <c r="B57" s="29" t="n"/>
-      <c r="C57" s="29" t="n"/>
-      <c r="D57" s="29" t="n"/>
-      <c r="E57" s="30" t="n"/>
-      <c r="F57" s="29">
+      <c r="A57" s="39" t="n"/>
+      <c r="B57" s="40" t="n"/>
+      <c r="C57" s="40" t="n"/>
+      <c r="D57" s="40" t="n"/>
+      <c r="E57" s="41" t="n"/>
+      <c r="F57" s="40">
         <f>IF(D57&lt;&gt;"Saída","",IF(E57&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B57,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3582,12 +4341,12 @@
       <c r="H57" s="2" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" s="28" t="n"/>
-      <c r="B58" s="29" t="n"/>
-      <c r="C58" s="29" t="n"/>
-      <c r="D58" s="29" t="n"/>
-      <c r="E58" s="30" t="n"/>
-      <c r="F58" s="29">
+      <c r="A58" s="39" t="n"/>
+      <c r="B58" s="40" t="n"/>
+      <c r="C58" s="40" t="n"/>
+      <c r="D58" s="40" t="n"/>
+      <c r="E58" s="41" t="n"/>
+      <c r="F58" s="40">
         <f>IF(D58&lt;&gt;"Saída","",IF(E58&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B58,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3595,12 +4354,12 @@
       <c r="H58" s="2" t="n"/>
     </row>
     <row r="59">
-      <c r="A59" s="28" t="n"/>
-      <c r="B59" s="29" t="n"/>
-      <c r="C59" s="29" t="n"/>
-      <c r="D59" s="29" t="n"/>
-      <c r="E59" s="30" t="n"/>
-      <c r="F59" s="29">
+      <c r="A59" s="39" t="n"/>
+      <c r="B59" s="40" t="n"/>
+      <c r="C59" s="40" t="n"/>
+      <c r="D59" s="40" t="n"/>
+      <c r="E59" s="41" t="n"/>
+      <c r="F59" s="40">
         <f>IF(D59&lt;&gt;"Saída","",IF(E59&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B59,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3608,12 +4367,12 @@
       <c r="H59" s="2" t="n"/>
     </row>
     <row r="60">
-      <c r="A60" s="28" t="n"/>
-      <c r="B60" s="29" t="n"/>
-      <c r="C60" s="29" t="n"/>
-      <c r="D60" s="29" t="n"/>
-      <c r="E60" s="30" t="n"/>
-      <c r="F60" s="29">
+      <c r="A60" s="39" t="n"/>
+      <c r="B60" s="40" t="n"/>
+      <c r="C60" s="40" t="n"/>
+      <c r="D60" s="40" t="n"/>
+      <c r="E60" s="41" t="n"/>
+      <c r="F60" s="40">
         <f>IF(D60&lt;&gt;"Saída","",IF(E60&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B60,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3621,12 +4380,12 @@
       <c r="H60" s="2" t="n"/>
     </row>
     <row r="61">
-      <c r="A61" s="28" t="n"/>
-      <c r="B61" s="29" t="n"/>
-      <c r="C61" s="29" t="n"/>
-      <c r="D61" s="29" t="n"/>
-      <c r="E61" s="30" t="n"/>
-      <c r="F61" s="29">
+      <c r="A61" s="39" t="n"/>
+      <c r="B61" s="40" t="n"/>
+      <c r="C61" s="40" t="n"/>
+      <c r="D61" s="40" t="n"/>
+      <c r="E61" s="41" t="n"/>
+      <c r="F61" s="40">
         <f>IF(D61&lt;&gt;"Saída","",IF(E61&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B61,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3634,12 +4393,12 @@
       <c r="H61" s="2" t="n"/>
     </row>
     <row r="62">
-      <c r="A62" s="28" t="n"/>
-      <c r="B62" s="29" t="n"/>
-      <c r="C62" s="29" t="n"/>
-      <c r="D62" s="29" t="n"/>
-      <c r="E62" s="30" t="n"/>
-      <c r="F62" s="29">
+      <c r="A62" s="39" t="n"/>
+      <c r="B62" s="40" t="n"/>
+      <c r="C62" s="40" t="n"/>
+      <c r="D62" s="40" t="n"/>
+      <c r="E62" s="41" t="n"/>
+      <c r="F62" s="40">
         <f>IF(D62&lt;&gt;"Saída","",IF(E62&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B62,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3647,12 +4406,12 @@
       <c r="H62" s="2" t="n"/>
     </row>
     <row r="63">
-      <c r="A63" s="28" t="n"/>
-      <c r="B63" s="29" t="n"/>
-      <c r="C63" s="29" t="n"/>
-      <c r="D63" s="29" t="n"/>
-      <c r="E63" s="30" t="n"/>
-      <c r="F63" s="29">
+      <c r="A63" s="39" t="n"/>
+      <c r="B63" s="40" t="n"/>
+      <c r="C63" s="40" t="n"/>
+      <c r="D63" s="40" t="n"/>
+      <c r="E63" s="41" t="n"/>
+      <c r="F63" s="40">
         <f>IF(D63&lt;&gt;"Saída","",IF(E63&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B63,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3660,12 +4419,12 @@
       <c r="H63" s="2" t="n"/>
     </row>
     <row r="64">
-      <c r="A64" s="28" t="n"/>
-      <c r="B64" s="29" t="n"/>
-      <c r="C64" s="29" t="n"/>
-      <c r="D64" s="29" t="n"/>
-      <c r="E64" s="30" t="n"/>
-      <c r="F64" s="29">
+      <c r="A64" s="39" t="n"/>
+      <c r="B64" s="40" t="n"/>
+      <c r="C64" s="40" t="n"/>
+      <c r="D64" s="40" t="n"/>
+      <c r="E64" s="41" t="n"/>
+      <c r="F64" s="40">
         <f>IF(D64&lt;&gt;"Saída","",IF(E64&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B64,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3673,12 +4432,12 @@
       <c r="H64" s="2" t="n"/>
     </row>
     <row r="65">
-      <c r="A65" s="28" t="n"/>
-      <c r="B65" s="29" t="n"/>
-      <c r="C65" s="29" t="n"/>
-      <c r="D65" s="29" t="n"/>
-      <c r="E65" s="30" t="n"/>
-      <c r="F65" s="29">
+      <c r="A65" s="39" t="n"/>
+      <c r="B65" s="40" t="n"/>
+      <c r="C65" s="40" t="n"/>
+      <c r="D65" s="40" t="n"/>
+      <c r="E65" s="41" t="n"/>
+      <c r="F65" s="40">
         <f>IF(D65&lt;&gt;"Saída","",IF(E65&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B65,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3686,12 +4445,12 @@
       <c r="H65" s="2" t="n"/>
     </row>
     <row r="66">
-      <c r="A66" s="28" t="n"/>
-      <c r="B66" s="29" t="n"/>
-      <c r="C66" s="29" t="n"/>
-      <c r="D66" s="29" t="n"/>
-      <c r="E66" s="30" t="n"/>
-      <c r="F66" s="29">
+      <c r="A66" s="39" t="n"/>
+      <c r="B66" s="40" t="n"/>
+      <c r="C66" s="40" t="n"/>
+      <c r="D66" s="40" t="n"/>
+      <c r="E66" s="41" t="n"/>
+      <c r="F66" s="40">
         <f>IF(D66&lt;&gt;"Saída","",IF(E66&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B66,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3699,12 +4458,12 @@
       <c r="H66" s="2" t="n"/>
     </row>
     <row r="67">
-      <c r="A67" s="28" t="n"/>
-      <c r="B67" s="29" t="n"/>
-      <c r="C67" s="29" t="n"/>
-      <c r="D67" s="29" t="n"/>
-      <c r="E67" s="30" t="n"/>
-      <c r="F67" s="29">
+      <c r="A67" s="39" t="n"/>
+      <c r="B67" s="40" t="n"/>
+      <c r="C67" s="40" t="n"/>
+      <c r="D67" s="40" t="n"/>
+      <c r="E67" s="41" t="n"/>
+      <c r="F67" s="40">
         <f>IF(D67&lt;&gt;"Saída","",IF(E67&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B67,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3712,12 +4471,12 @@
       <c r="H67" s="2" t="n"/>
     </row>
     <row r="68">
-      <c r="A68" s="28" t="n"/>
-      <c r="B68" s="29" t="n"/>
-      <c r="C68" s="29" t="n"/>
-      <c r="D68" s="29" t="n"/>
-      <c r="E68" s="30" t="n"/>
-      <c r="F68" s="29">
+      <c r="A68" s="39" t="n"/>
+      <c r="B68" s="40" t="n"/>
+      <c r="C68" s="40" t="n"/>
+      <c r="D68" s="40" t="n"/>
+      <c r="E68" s="41" t="n"/>
+      <c r="F68" s="40">
         <f>IF(D68&lt;&gt;"Saída","",IF(E68&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B68,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3725,12 +4484,12 @@
       <c r="H68" s="2" t="n"/>
     </row>
     <row r="69">
-      <c r="A69" s="28" t="n"/>
-      <c r="B69" s="29" t="n"/>
-      <c r="C69" s="29" t="n"/>
-      <c r="D69" s="29" t="n"/>
-      <c r="E69" s="30" t="n"/>
-      <c r="F69" s="29">
+      <c r="A69" s="39" t="n"/>
+      <c r="B69" s="40" t="n"/>
+      <c r="C69" s="40" t="n"/>
+      <c r="D69" s="40" t="n"/>
+      <c r="E69" s="41" t="n"/>
+      <c r="F69" s="40">
         <f>IF(D69&lt;&gt;"Saída","",IF(E69&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B69,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3738,12 +4497,12 @@
       <c r="H69" s="2" t="n"/>
     </row>
     <row r="70">
-      <c r="A70" s="28" t="n"/>
-      <c r="B70" s="29" t="n"/>
-      <c r="C70" s="29" t="n"/>
-      <c r="D70" s="29" t="n"/>
-      <c r="E70" s="30" t="n"/>
-      <c r="F70" s="29">
+      <c r="A70" s="39" t="n"/>
+      <c r="B70" s="40" t="n"/>
+      <c r="C70" s="40" t="n"/>
+      <c r="D70" s="40" t="n"/>
+      <c r="E70" s="41" t="n"/>
+      <c r="F70" s="40">
         <f>IF(D70&lt;&gt;"Saída","",IF(E70&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B70,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3751,12 +4510,12 @@
       <c r="H70" s="2" t="n"/>
     </row>
     <row r="71">
-      <c r="A71" s="28" t="n"/>
-      <c r="B71" s="29" t="n"/>
-      <c r="C71" s="29" t="n"/>
-      <c r="D71" s="29" t="n"/>
-      <c r="E71" s="30" t="n"/>
-      <c r="F71" s="29">
+      <c r="A71" s="39" t="n"/>
+      <c r="B71" s="40" t="n"/>
+      <c r="C71" s="40" t="n"/>
+      <c r="D71" s="40" t="n"/>
+      <c r="E71" s="41" t="n"/>
+      <c r="F71" s="40">
         <f>IF(D71&lt;&gt;"Saída","",IF(E71&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B71,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3764,12 +4523,12 @@
       <c r="H71" s="2" t="n"/>
     </row>
     <row r="72">
-      <c r="A72" s="28" t="n"/>
-      <c r="B72" s="29" t="n"/>
-      <c r="C72" s="29" t="n"/>
-      <c r="D72" s="29" t="n"/>
-      <c r="E72" s="30" t="n"/>
-      <c r="F72" s="29">
+      <c r="A72" s="39" t="n"/>
+      <c r="B72" s="40" t="n"/>
+      <c r="C72" s="40" t="n"/>
+      <c r="D72" s="40" t="n"/>
+      <c r="E72" s="41" t="n"/>
+      <c r="F72" s="40">
         <f>IF(D72&lt;&gt;"Saída","",IF(E72&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B72,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3777,12 +4536,12 @@
       <c r="H72" s="2" t="n"/>
     </row>
     <row r="73">
-      <c r="A73" s="28" t="n"/>
-      <c r="B73" s="29" t="n"/>
-      <c r="C73" s="29" t="n"/>
-      <c r="D73" s="29" t="n"/>
-      <c r="E73" s="30" t="n"/>
-      <c r="F73" s="29">
+      <c r="A73" s="39" t="n"/>
+      <c r="B73" s="40" t="n"/>
+      <c r="C73" s="40" t="n"/>
+      <c r="D73" s="40" t="n"/>
+      <c r="E73" s="41" t="n"/>
+      <c r="F73" s="40">
         <f>IF(D73&lt;&gt;"Saída","",IF(E73&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B73,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3790,12 +4549,12 @@
       <c r="H73" s="2" t="n"/>
     </row>
     <row r="74">
-      <c r="A74" s="28" t="n"/>
-      <c r="B74" s="29" t="n"/>
-      <c r="C74" s="29" t="n"/>
-      <c r="D74" s="29" t="n"/>
-      <c r="E74" s="30" t="n"/>
-      <c r="F74" s="29">
+      <c r="A74" s="39" t="n"/>
+      <c r="B74" s="40" t="n"/>
+      <c r="C74" s="40" t="n"/>
+      <c r="D74" s="40" t="n"/>
+      <c r="E74" s="41" t="n"/>
+      <c r="F74" s="40">
         <f>IF(D74&lt;&gt;"Saída","",IF(E74&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B74,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3803,12 +4562,12 @@
       <c r="H74" s="2" t="n"/>
     </row>
     <row r="75">
-      <c r="A75" s="28" t="n"/>
-      <c r="B75" s="29" t="n"/>
-      <c r="C75" s="29" t="n"/>
-      <c r="D75" s="29" t="n"/>
-      <c r="E75" s="30" t="n"/>
-      <c r="F75" s="29">
+      <c r="A75" s="39" t="n"/>
+      <c r="B75" s="40" t="n"/>
+      <c r="C75" s="40" t="n"/>
+      <c r="D75" s="40" t="n"/>
+      <c r="E75" s="41" t="n"/>
+      <c r="F75" s="40">
         <f>IF(D75&lt;&gt;"Saída","",IF(E75&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B75,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3816,12 +4575,12 @@
       <c r="H75" s="2" t="n"/>
     </row>
     <row r="76">
-      <c r="A76" s="28" t="n"/>
-      <c r="B76" s="29" t="n"/>
-      <c r="C76" s="29" t="n"/>
-      <c r="D76" s="29" t="n"/>
-      <c r="E76" s="30" t="n"/>
-      <c r="F76" s="29">
+      <c r="A76" s="39" t="n"/>
+      <c r="B76" s="40" t="n"/>
+      <c r="C76" s="40" t="n"/>
+      <c r="D76" s="40" t="n"/>
+      <c r="E76" s="41" t="n"/>
+      <c r="F76" s="40">
         <f>IF(D76&lt;&gt;"Saída","",IF(E76&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B76,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3829,12 +4588,12 @@
       <c r="H76" s="2" t="n"/>
     </row>
     <row r="77">
-      <c r="A77" s="28" t="n"/>
-      <c r="B77" s="29" t="n"/>
-      <c r="C77" s="29" t="n"/>
-      <c r="D77" s="29" t="n"/>
-      <c r="E77" s="30" t="n"/>
-      <c r="F77" s="29">
+      <c r="A77" s="39" t="n"/>
+      <c r="B77" s="40" t="n"/>
+      <c r="C77" s="40" t="n"/>
+      <c r="D77" s="40" t="n"/>
+      <c r="E77" s="41" t="n"/>
+      <c r="F77" s="40">
         <f>IF(D77&lt;&gt;"Saída","",IF(E77&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B77,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3842,12 +4601,12 @@
       <c r="H77" s="2" t="n"/>
     </row>
     <row r="78">
-      <c r="A78" s="28" t="n"/>
-      <c r="B78" s="29" t="n"/>
-      <c r="C78" s="29" t="n"/>
-      <c r="D78" s="29" t="n"/>
-      <c r="E78" s="30" t="n"/>
-      <c r="F78" s="29">
+      <c r="A78" s="39" t="n"/>
+      <c r="B78" s="40" t="n"/>
+      <c r="C78" s="40" t="n"/>
+      <c r="D78" s="40" t="n"/>
+      <c r="E78" s="41" t="n"/>
+      <c r="F78" s="40">
         <f>IF(D78&lt;&gt;"Saída","",IF(E78&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B78,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3855,12 +4614,12 @@
       <c r="H78" s="2" t="n"/>
     </row>
     <row r="79">
-      <c r="A79" s="28" t="n"/>
-      <c r="B79" s="29" t="n"/>
-      <c r="C79" s="29" t="n"/>
-      <c r="D79" s="29" t="n"/>
-      <c r="E79" s="30" t="n"/>
-      <c r="F79" s="29">
+      <c r="A79" s="39" t="n"/>
+      <c r="B79" s="40" t="n"/>
+      <c r="C79" s="40" t="n"/>
+      <c r="D79" s="40" t="n"/>
+      <c r="E79" s="41" t="n"/>
+      <c r="F79" s="40">
         <f>IF(D79&lt;&gt;"Saída","",IF(E79&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B79,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3868,12 +4627,12 @@
       <c r="H79" s="2" t="n"/>
     </row>
     <row r="80">
-      <c r="A80" s="28" t="n"/>
-      <c r="B80" s="29" t="n"/>
-      <c r="C80" s="29" t="n"/>
-      <c r="D80" s="29" t="n"/>
-      <c r="E80" s="30" t="n"/>
-      <c r="F80" s="29">
+      <c r="A80" s="39" t="n"/>
+      <c r="B80" s="40" t="n"/>
+      <c r="C80" s="40" t="n"/>
+      <c r="D80" s="40" t="n"/>
+      <c r="E80" s="41" t="n"/>
+      <c r="F80" s="40">
         <f>IF(D80&lt;&gt;"Saída","",IF(E80&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B80,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3881,12 +4640,12 @@
       <c r="H80" s="2" t="n"/>
     </row>
     <row r="81">
-      <c r="A81" s="28" t="n"/>
-      <c r="B81" s="29" t="n"/>
-      <c r="C81" s="29" t="n"/>
-      <c r="D81" s="29" t="n"/>
-      <c r="E81" s="30" t="n"/>
-      <c r="F81" s="29">
+      <c r="A81" s="39" t="n"/>
+      <c r="B81" s="40" t="n"/>
+      <c r="C81" s="40" t="n"/>
+      <c r="D81" s="40" t="n"/>
+      <c r="E81" s="41" t="n"/>
+      <c r="F81" s="40">
         <f>IF(D81&lt;&gt;"Saída","",IF(E81&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B81,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3894,12 +4653,12 @@
       <c r="H81" s="2" t="n"/>
     </row>
     <row r="82">
-      <c r="A82" s="28" t="n"/>
-      <c r="B82" s="29" t="n"/>
-      <c r="C82" s="29" t="n"/>
-      <c r="D82" s="29" t="n"/>
-      <c r="E82" s="30" t="n"/>
-      <c r="F82" s="29">
+      <c r="A82" s="39" t="n"/>
+      <c r="B82" s="40" t="n"/>
+      <c r="C82" s="40" t="n"/>
+      <c r="D82" s="40" t="n"/>
+      <c r="E82" s="41" t="n"/>
+      <c r="F82" s="40">
         <f>IF(D82&lt;&gt;"Saída","",IF(E82&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B82,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3907,12 +4666,12 @@
       <c r="H82" s="2" t="n"/>
     </row>
     <row r="83">
-      <c r="A83" s="28" t="n"/>
-      <c r="B83" s="29" t="n"/>
-      <c r="C83" s="29" t="n"/>
-      <c r="D83" s="29" t="n"/>
-      <c r="E83" s="30" t="n"/>
-      <c r="F83" s="29">
+      <c r="A83" s="39" t="n"/>
+      <c r="B83" s="40" t="n"/>
+      <c r="C83" s="40" t="n"/>
+      <c r="D83" s="40" t="n"/>
+      <c r="E83" s="41" t="n"/>
+      <c r="F83" s="40">
         <f>IF(D83&lt;&gt;"Saída","",IF(E83&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B83,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3920,12 +4679,12 @@
       <c r="H83" s="2" t="n"/>
     </row>
     <row r="84">
-      <c r="A84" s="28" t="n"/>
-      <c r="B84" s="29" t="n"/>
-      <c r="C84" s="29" t="n"/>
-      <c r="D84" s="29" t="n"/>
-      <c r="E84" s="30" t="n"/>
-      <c r="F84" s="29">
+      <c r="A84" s="39" t="n"/>
+      <c r="B84" s="40" t="n"/>
+      <c r="C84" s="40" t="n"/>
+      <c r="D84" s="40" t="n"/>
+      <c r="E84" s="41" t="n"/>
+      <c r="F84" s="40">
         <f>IF(D84&lt;&gt;"Saída","",IF(E84&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B84,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3933,12 +4692,12 @@
       <c r="H84" s="2" t="n"/>
     </row>
     <row r="85">
-      <c r="A85" s="28" t="n"/>
-      <c r="B85" s="29" t="n"/>
-      <c r="C85" s="29" t="n"/>
-      <c r="D85" s="29" t="n"/>
-      <c r="E85" s="30" t="n"/>
-      <c r="F85" s="29">
+      <c r="A85" s="39" t="n"/>
+      <c r="B85" s="40" t="n"/>
+      <c r="C85" s="40" t="n"/>
+      <c r="D85" s="40" t="n"/>
+      <c r="E85" s="41" t="n"/>
+      <c r="F85" s="40">
         <f>IF(D85&lt;&gt;"Saída","",IF(E85&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B85,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3946,12 +4705,12 @@
       <c r="H85" s="2" t="n"/>
     </row>
     <row r="86">
-      <c r="A86" s="28" t="n"/>
-      <c r="B86" s="29" t="n"/>
-      <c r="C86" s="29" t="n"/>
-      <c r="D86" s="29" t="n"/>
-      <c r="E86" s="30" t="n"/>
-      <c r="F86" s="29">
+      <c r="A86" s="39" t="n"/>
+      <c r="B86" s="40" t="n"/>
+      <c r="C86" s="40" t="n"/>
+      <c r="D86" s="40" t="n"/>
+      <c r="E86" s="41" t="n"/>
+      <c r="F86" s="40">
         <f>IF(D86&lt;&gt;"Saída","",IF(E86&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B86,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3959,12 +4718,12 @@
       <c r="H86" s="2" t="n"/>
     </row>
     <row r="87">
-      <c r="A87" s="28" t="n"/>
-      <c r="B87" s="29" t="n"/>
-      <c r="C87" s="29" t="n"/>
-      <c r="D87" s="29" t="n"/>
-      <c r="E87" s="30" t="n"/>
-      <c r="F87" s="29">
+      <c r="A87" s="39" t="n"/>
+      <c r="B87" s="40" t="n"/>
+      <c r="C87" s="40" t="n"/>
+      <c r="D87" s="40" t="n"/>
+      <c r="E87" s="41" t="n"/>
+      <c r="F87" s="40">
         <f>IF(D87&lt;&gt;"Saída","",IF(E87&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B87,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3972,12 +4731,12 @@
       <c r="H87" s="2" t="n"/>
     </row>
     <row r="88">
-      <c r="A88" s="28" t="n"/>
-      <c r="B88" s="29" t="n"/>
-      <c r="C88" s="29" t="n"/>
-      <c r="D88" s="29" t="n"/>
-      <c r="E88" s="30" t="n"/>
-      <c r="F88" s="29">
+      <c r="A88" s="39" t="n"/>
+      <c r="B88" s="40" t="n"/>
+      <c r="C88" s="40" t="n"/>
+      <c r="D88" s="40" t="n"/>
+      <c r="E88" s="41" t="n"/>
+      <c r="F88" s="40">
         <f>IF(D88&lt;&gt;"Saída","",IF(E88&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B88,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3985,12 +4744,12 @@
       <c r="H88" s="2" t="n"/>
     </row>
     <row r="89">
-      <c r="A89" s="28" t="n"/>
-      <c r="B89" s="29" t="n"/>
-      <c r="C89" s="29" t="n"/>
-      <c r="D89" s="29" t="n"/>
-      <c r="E89" s="30" t="n"/>
-      <c r="F89" s="29">
+      <c r="A89" s="39" t="n"/>
+      <c r="B89" s="40" t="n"/>
+      <c r="C89" s="40" t="n"/>
+      <c r="D89" s="40" t="n"/>
+      <c r="E89" s="41" t="n"/>
+      <c r="F89" s="40">
         <f>IF(D89&lt;&gt;"Saída","",IF(E89&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B89,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -3998,12 +4757,12 @@
       <c r="H89" s="2" t="n"/>
     </row>
     <row r="90">
-      <c r="A90" s="28" t="n"/>
-      <c r="B90" s="29" t="n"/>
-      <c r="C90" s="29" t="n"/>
-      <c r="D90" s="29" t="n"/>
-      <c r="E90" s="30" t="n"/>
-      <c r="F90" s="29">
+      <c r="A90" s="39" t="n"/>
+      <c r="B90" s="40" t="n"/>
+      <c r="C90" s="40" t="n"/>
+      <c r="D90" s="40" t="n"/>
+      <c r="E90" s="41" t="n"/>
+      <c r="F90" s="40">
         <f>IF(D90&lt;&gt;"Saída","",IF(E90&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B90,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -4011,12 +4770,12 @@
       <c r="H90" s="2" t="n"/>
     </row>
     <row r="91">
-      <c r="A91" s="28" t="n"/>
-      <c r="B91" s="29" t="n"/>
-      <c r="C91" s="29" t="n"/>
-      <c r="D91" s="29" t="n"/>
-      <c r="E91" s="30" t="n"/>
-      <c r="F91" s="29">
+      <c r="A91" s="39" t="n"/>
+      <c r="B91" s="40" t="n"/>
+      <c r="C91" s="40" t="n"/>
+      <c r="D91" s="40" t="n"/>
+      <c r="E91" s="41" t="n"/>
+      <c r="F91" s="40">
         <f>IF(D91&lt;&gt;"Saída","",IF(E91&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B91,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -4024,12 +4783,12 @@
       <c r="H91" s="2" t="n"/>
     </row>
     <row r="92">
-      <c r="A92" s="28" t="n"/>
-      <c r="B92" s="29" t="n"/>
-      <c r="C92" s="29" t="n"/>
-      <c r="D92" s="29" t="n"/>
-      <c r="E92" s="30" t="n"/>
-      <c r="F92" s="29">
+      <c r="A92" s="39" t="n"/>
+      <c r="B92" s="40" t="n"/>
+      <c r="C92" s="40" t="n"/>
+      <c r="D92" s="40" t="n"/>
+      <c r="E92" s="41" t="n"/>
+      <c r="F92" s="40">
         <f>IF(D92&lt;&gt;"Saída","",IF(E92&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B92,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -4037,12 +4796,12 @@
       <c r="H92" s="2" t="n"/>
     </row>
     <row r="93">
-      <c r="A93" s="28" t="n"/>
-      <c r="B93" s="29" t="n"/>
-      <c r="C93" s="29" t="n"/>
-      <c r="D93" s="29" t="n"/>
-      <c r="E93" s="30" t="n"/>
-      <c r="F93" s="29">
+      <c r="A93" s="39" t="n"/>
+      <c r="B93" s="40" t="n"/>
+      <c r="C93" s="40" t="n"/>
+      <c r="D93" s="40" t="n"/>
+      <c r="E93" s="41" t="n"/>
+      <c r="F93" s="40">
         <f>IF(D93&lt;&gt;"Saída","",IF(E93&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B93,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -4050,12 +4809,12 @@
       <c r="H93" s="2" t="n"/>
     </row>
     <row r="94">
-      <c r="A94" s="28" t="n"/>
-      <c r="B94" s="29" t="n"/>
-      <c r="C94" s="29" t="n"/>
-      <c r="D94" s="29" t="n"/>
-      <c r="E94" s="30" t="n"/>
-      <c r="F94" s="29">
+      <c r="A94" s="39" t="n"/>
+      <c r="B94" s="40" t="n"/>
+      <c r="C94" s="40" t="n"/>
+      <c r="D94" s="40" t="n"/>
+      <c r="E94" s="41" t="n"/>
+      <c r="F94" s="40">
         <f>IF(D94&lt;&gt;"Saída","",IF(E94&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B94,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -4063,12 +4822,12 @@
       <c r="H94" s="2" t="n"/>
     </row>
     <row r="95">
-      <c r="A95" s="28" t="n"/>
-      <c r="B95" s="29" t="n"/>
-      <c r="C95" s="29" t="n"/>
-      <c r="D95" s="29" t="n"/>
-      <c r="E95" s="30" t="n"/>
-      <c r="F95" s="29">
+      <c r="A95" s="39" t="n"/>
+      <c r="B95" s="40" t="n"/>
+      <c r="C95" s="40" t="n"/>
+      <c r="D95" s="40" t="n"/>
+      <c r="E95" s="41" t="n"/>
+      <c r="F95" s="40">
         <f>IF(D95&lt;&gt;"Saída","",IF(E95&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B95,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -4076,12 +4835,12 @@
       <c r="H95" s="2" t="n"/>
     </row>
     <row r="96">
-      <c r="A96" s="28" t="n"/>
-      <c r="B96" s="29" t="n"/>
-      <c r="C96" s="29" t="n"/>
-      <c r="D96" s="29" t="n"/>
-      <c r="E96" s="30" t="n"/>
-      <c r="F96" s="29">
+      <c r="A96" s="39" t="n"/>
+      <c r="B96" s="40" t="n"/>
+      <c r="C96" s="40" t="n"/>
+      <c r="D96" s="40" t="n"/>
+      <c r="E96" s="41" t="n"/>
+      <c r="F96" s="40">
         <f>IF(D96&lt;&gt;"Saída","",IF(E96&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B96,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -4089,12 +4848,12 @@
       <c r="H96" s="2" t="n"/>
     </row>
     <row r="97">
-      <c r="A97" s="28" t="n"/>
-      <c r="B97" s="29" t="n"/>
-      <c r="C97" s="29" t="n"/>
-      <c r="D97" s="29" t="n"/>
-      <c r="E97" s="30" t="n"/>
-      <c r="F97" s="29">
+      <c r="A97" s="39" t="n"/>
+      <c r="B97" s="40" t="n"/>
+      <c r="C97" s="40" t="n"/>
+      <c r="D97" s="40" t="n"/>
+      <c r="E97" s="41" t="n"/>
+      <c r="F97" s="40">
         <f>IF(D97&lt;&gt;"Saída","",IF(E97&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B97,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -4102,12 +4861,12 @@
       <c r="H97" s="2" t="n"/>
     </row>
     <row r="98">
-      <c r="A98" s="28" t="n"/>
-      <c r="B98" s="29" t="n"/>
-      <c r="C98" s="29" t="n"/>
-      <c r="D98" s="29" t="n"/>
-      <c r="E98" s="30" t="n"/>
-      <c r="F98" s="29">
+      <c r="A98" s="39" t="n"/>
+      <c r="B98" s="40" t="n"/>
+      <c r="C98" s="40" t="n"/>
+      <c r="D98" s="40" t="n"/>
+      <c r="E98" s="41" t="n"/>
+      <c r="F98" s="40">
         <f>IF(D98&lt;&gt;"Saída","",IF(E98&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B98,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -4115,12 +4874,12 @@
       <c r="H98" s="2" t="n"/>
     </row>
     <row r="99">
-      <c r="A99" s="28" t="n"/>
-      <c r="B99" s="29" t="n"/>
-      <c r="C99" s="29" t="n"/>
-      <c r="D99" s="29" t="n"/>
-      <c r="E99" s="30" t="n"/>
-      <c r="F99" s="29">
+      <c r="A99" s="39" t="n"/>
+      <c r="B99" s="40" t="n"/>
+      <c r="C99" s="40" t="n"/>
+      <c r="D99" s="40" t="n"/>
+      <c r="E99" s="41" t="n"/>
+      <c r="F99" s="40">
         <f>IF(D99&lt;&gt;"Saída","",IF(E99&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B99,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -4128,12 +4887,12 @@
       <c r="H99" s="2" t="n"/>
     </row>
     <row r="100">
-      <c r="A100" s="28" t="n"/>
-      <c r="B100" s="29" t="n"/>
-      <c r="C100" s="29" t="n"/>
-      <c r="D100" s="29" t="n"/>
-      <c r="E100" s="30" t="n"/>
-      <c r="F100" s="29">
+      <c r="A100" s="39" t="n"/>
+      <c r="B100" s="40" t="n"/>
+      <c r="C100" s="40" t="n"/>
+      <c r="D100" s="40" t="n"/>
+      <c r="E100" s="41" t="n"/>
+      <c r="F100" s="40">
         <f>IF(D100&lt;&gt;"Saída","",IF(E100&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B100,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -4141,12 +4900,12 @@
       <c r="H100" s="2" t="n"/>
     </row>
     <row r="101">
-      <c r="A101" s="28" t="n"/>
-      <c r="B101" s="29" t="n"/>
-      <c r="C101" s="29" t="n"/>
-      <c r="D101" s="29" t="n"/>
-      <c r="E101" s="30" t="n"/>
-      <c r="F101" s="29">
+      <c r="A101" s="39" t="n"/>
+      <c r="B101" s="40" t="n"/>
+      <c r="C101" s="40" t="n"/>
+      <c r="D101" s="40" t="n"/>
+      <c r="E101" s="41" t="n"/>
+      <c r="F101" s="40">
         <f>IF(D101&lt;&gt;"Saída","",IF(E101&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B101,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -4154,12 +4913,12 @@
       <c r="H101" s="2" t="n"/>
     </row>
     <row r="102">
-      <c r="A102" s="28" t="n"/>
-      <c r="B102" s="29" t="n"/>
-      <c r="C102" s="29" t="n"/>
-      <c r="D102" s="29" t="n"/>
-      <c r="E102" s="30" t="n"/>
-      <c r="F102" s="29">
+      <c r="A102" s="39" t="n"/>
+      <c r="B102" s="40" t="n"/>
+      <c r="C102" s="40" t="n"/>
+      <c r="D102" s="40" t="n"/>
+      <c r="E102" s="41" t="n"/>
+      <c r="F102" s="40">
         <f>IF(D102&lt;&gt;"Saída","",IF(E102&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B102,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -4167,12 +4926,12 @@
       <c r="H102" s="2" t="n"/>
     </row>
     <row r="103">
-      <c r="A103" s="28" t="n"/>
-      <c r="B103" s="29" t="n"/>
-      <c r="C103" s="29" t="n"/>
-      <c r="D103" s="29" t="n"/>
-      <c r="E103" s="30" t="n"/>
-      <c r="F103" s="29">
+      <c r="A103" s="39" t="n"/>
+      <c r="B103" s="40" t="n"/>
+      <c r="C103" s="40" t="n"/>
+      <c r="D103" s="40" t="n"/>
+      <c r="E103" s="41" t="n"/>
+      <c r="F103" s="40">
         <f>IF(D103&lt;&gt;"Saída","",IF(E103&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B103,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -4180,12 +4939,12 @@
       <c r="H103" s="2" t="n"/>
     </row>
     <row r="104">
-      <c r="A104" s="28" t="n"/>
-      <c r="B104" s="29" t="n"/>
-      <c r="C104" s="29" t="n"/>
-      <c r="D104" s="29" t="n"/>
-      <c r="E104" s="30" t="n"/>
-      <c r="F104" s="29">
+      <c r="A104" s="39" t="n"/>
+      <c r="B104" s="40" t="n"/>
+      <c r="C104" s="40" t="n"/>
+      <c r="D104" s="40" t="n"/>
+      <c r="E104" s="41" t="n"/>
+      <c r="F104" s="40">
         <f>IF(D104&lt;&gt;"Saída","",IF(E104&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B104,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -4193,12 +4952,12 @@
       <c r="H104" s="2" t="n"/>
     </row>
     <row r="105">
-      <c r="A105" s="28" t="n"/>
-      <c r="B105" s="29" t="n"/>
-      <c r="C105" s="29" t="n"/>
-      <c r="D105" s="29" t="n"/>
-      <c r="E105" s="30" t="n"/>
-      <c r="F105" s="29">
+      <c r="A105" s="39" t="n"/>
+      <c r="B105" s="40" t="n"/>
+      <c r="C105" s="40" t="n"/>
+      <c r="D105" s="40" t="n"/>
+      <c r="E105" s="41" t="n"/>
+      <c r="F105" s="40">
         <f>IF(D105&lt;&gt;"Saída","",IF(E105&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B105,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -4206,12 +4965,12 @@
       <c r="H105" s="2" t="n"/>
     </row>
     <row r="106">
-      <c r="A106" s="28" t="n"/>
-      <c r="B106" s="29" t="n"/>
-      <c r="C106" s="29" t="n"/>
-      <c r="D106" s="29" t="n"/>
-      <c r="E106" s="30" t="n"/>
-      <c r="F106" s="29">
+      <c r="A106" s="39" t="n"/>
+      <c r="B106" s="40" t="n"/>
+      <c r="C106" s="40" t="n"/>
+      <c r="D106" s="40" t="n"/>
+      <c r="E106" s="41" t="n"/>
+      <c r="F106" s="40">
         <f>IF(D106&lt;&gt;"Saída","",IF(E106&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B106,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -4219,12 +4978,12 @@
       <c r="H106" s="2" t="n"/>
     </row>
     <row r="107">
-      <c r="A107" s="28" t="n"/>
-      <c r="B107" s="29" t="n"/>
-      <c r="C107" s="29" t="n"/>
-      <c r="D107" s="29" t="n"/>
-      <c r="E107" s="30" t="n"/>
-      <c r="F107" s="29">
+      <c r="A107" s="39" t="n"/>
+      <c r="B107" s="40" t="n"/>
+      <c r="C107" s="40" t="n"/>
+      <c r="D107" s="40" t="n"/>
+      <c r="E107" s="41" t="n"/>
+      <c r="F107" s="40">
         <f>IF(D107&lt;&gt;"Saída","",IF(E107&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B107,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -4232,12 +4991,12 @@
       <c r="H107" s="2" t="n"/>
     </row>
     <row r="108">
-      <c r="A108" s="28" t="n"/>
-      <c r="B108" s="29" t="n"/>
-      <c r="C108" s="29" t="n"/>
-      <c r="D108" s="29" t="n"/>
-      <c r="E108" s="30" t="n"/>
-      <c r="F108" s="29">
+      <c r="A108" s="39" t="n"/>
+      <c r="B108" s="40" t="n"/>
+      <c r="C108" s="40" t="n"/>
+      <c r="D108" s="40" t="n"/>
+      <c r="E108" s="41" t="n"/>
+      <c r="F108" s="40">
         <f>IF(D108&lt;&gt;"Saída","",IF(E108&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B108,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -4245,12 +5004,12 @@
       <c r="H108" s="2" t="n"/>
     </row>
     <row r="109">
-      <c r="A109" s="28" t="n"/>
-      <c r="B109" s="29" t="n"/>
-      <c r="C109" s="29" t="n"/>
-      <c r="D109" s="29" t="n"/>
-      <c r="E109" s="30" t="n"/>
-      <c r="F109" s="29">
+      <c r="A109" s="39" t="n"/>
+      <c r="B109" s="40" t="n"/>
+      <c r="C109" s="40" t="n"/>
+      <c r="D109" s="40" t="n"/>
+      <c r="E109" s="41" t="n"/>
+      <c r="F109" s="40">
         <f>IF(D109&lt;&gt;"Saída","",IF(E109&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B109,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -4258,12 +5017,12 @@
       <c r="H109" s="2" t="n"/>
     </row>
     <row r="110">
-      <c r="A110" s="28" t="n"/>
-      <c r="B110" s="29" t="n"/>
-      <c r="C110" s="29" t="n"/>
-      <c r="D110" s="29" t="n"/>
-      <c r="E110" s="30" t="n"/>
-      <c r="F110" s="29">
+      <c r="A110" s="39" t="n"/>
+      <c r="B110" s="40" t="n"/>
+      <c r="C110" s="40" t="n"/>
+      <c r="D110" s="40" t="n"/>
+      <c r="E110" s="41" t="n"/>
+      <c r="F110" s="40">
         <f>IF(D110&lt;&gt;"Saída","",IF(E110&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B110,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -4271,12 +5030,12 @@
       <c r="H110" s="2" t="n"/>
     </row>
     <row r="111">
-      <c r="A111" s="28" t="n"/>
-      <c r="B111" s="29" t="n"/>
-      <c r="C111" s="29" t="n"/>
-      <c r="D111" s="29" t="n"/>
-      <c r="E111" s="30" t="n"/>
-      <c r="F111" s="29">
+      <c r="A111" s="39" t="n"/>
+      <c r="B111" s="40" t="n"/>
+      <c r="C111" s="40" t="n"/>
+      <c r="D111" s="40" t="n"/>
+      <c r="E111" s="41" t="n"/>
+      <c r="F111" s="40">
         <f>IF(D111&lt;&gt;"Saída","",IF(E111&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B111,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -4284,12 +5043,12 @@
       <c r="H111" s="2" t="n"/>
     </row>
     <row r="112">
-      <c r="A112" s="28" t="n"/>
-      <c r="B112" s="29" t="n"/>
-      <c r="C112" s="29" t="n"/>
-      <c r="D112" s="29" t="n"/>
-      <c r="E112" s="30" t="n"/>
-      <c r="F112" s="29">
+      <c r="A112" s="39" t="n"/>
+      <c r="B112" s="40" t="n"/>
+      <c r="C112" s="40" t="n"/>
+      <c r="D112" s="40" t="n"/>
+      <c r="E112" s="41" t="n"/>
+      <c r="F112" s="40">
         <f>IF(D112&lt;&gt;"Saída","",IF(E112&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B112,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -4297,12 +5056,12 @@
       <c r="H112" s="2" t="n"/>
     </row>
     <row r="113">
-      <c r="A113" s="28" t="n"/>
-      <c r="B113" s="29" t="n"/>
-      <c r="C113" s="29" t="n"/>
-      <c r="D113" s="29" t="n"/>
-      <c r="E113" s="30" t="n"/>
-      <c r="F113" s="29">
+      <c r="A113" s="39" t="n"/>
+      <c r="B113" s="40" t="n"/>
+      <c r="C113" s="40" t="n"/>
+      <c r="D113" s="40" t="n"/>
+      <c r="E113" s="41" t="n"/>
+      <c r="F113" s="40">
         <f>IF(D113&lt;&gt;"Saída","",IF(E113&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B113,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -4310,12 +5069,12 @@
       <c r="H113" s="2" t="n"/>
     </row>
     <row r="114">
-      <c r="A114" s="28" t="n"/>
-      <c r="B114" s="29" t="n"/>
-      <c r="C114" s="29" t="n"/>
-      <c r="D114" s="29" t="n"/>
-      <c r="E114" s="30" t="n"/>
-      <c r="F114" s="29">
+      <c r="A114" s="39" t="n"/>
+      <c r="B114" s="40" t="n"/>
+      <c r="C114" s="40" t="n"/>
+      <c r="D114" s="40" t="n"/>
+      <c r="E114" s="41" t="n"/>
+      <c r="F114" s="40">
         <f>IF(D114&lt;&gt;"Saída","",IF(E114&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B114,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -4323,12 +5082,12 @@
       <c r="H114" s="2" t="n"/>
     </row>
     <row r="115">
-      <c r="A115" s="28" t="n"/>
-      <c r="B115" s="29" t="n"/>
-      <c r="C115" s="29" t="n"/>
-      <c r="D115" s="29" t="n"/>
-      <c r="E115" s="30" t="n"/>
-      <c r="F115" s="29">
+      <c r="A115" s="39" t="n"/>
+      <c r="B115" s="40" t="n"/>
+      <c r="C115" s="40" t="n"/>
+      <c r="D115" s="40" t="n"/>
+      <c r="E115" s="41" t="n"/>
+      <c r="F115" s="40">
         <f>IF(D115&lt;&gt;"Saída","",IF(E115&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B115,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -4336,12 +5095,12 @@
       <c r="H115" s="2" t="n"/>
     </row>
     <row r="116">
-      <c r="A116" s="28" t="n"/>
-      <c r="B116" s="29" t="n"/>
-      <c r="C116" s="29" t="n"/>
-      <c r="D116" s="29" t="n"/>
-      <c r="E116" s="30" t="n"/>
-      <c r="F116" s="29">
+      <c r="A116" s="39" t="n"/>
+      <c r="B116" s="40" t="n"/>
+      <c r="C116" s="40" t="n"/>
+      <c r="D116" s="40" t="n"/>
+      <c r="E116" s="41" t="n"/>
+      <c r="F116" s="40">
         <f>IF(D116&lt;&gt;"Saída","",IF(E116&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B116,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -4349,12 +5108,12 @@
       <c r="H116" s="2" t="n"/>
     </row>
     <row r="117">
-      <c r="A117" s="28" t="n"/>
-      <c r="B117" s="29" t="n"/>
-      <c r="C117" s="29" t="n"/>
-      <c r="D117" s="29" t="n"/>
-      <c r="E117" s="30" t="n"/>
-      <c r="F117" s="29">
+      <c r="A117" s="39" t="n"/>
+      <c r="B117" s="40" t="n"/>
+      <c r="C117" s="40" t="n"/>
+      <c r="D117" s="40" t="n"/>
+      <c r="E117" s="41" t="n"/>
+      <c r="F117" s="40">
         <f>IF(D117&lt;&gt;"Saída","",IF(E117&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B117,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -4362,12 +5121,12 @@
       <c r="H117" s="2" t="n"/>
     </row>
     <row r="118">
-      <c r="A118" s="28" t="n"/>
-      <c r="B118" s="29" t="n"/>
-      <c r="C118" s="29" t="n"/>
-      <c r="D118" s="29" t="n"/>
-      <c r="E118" s="30" t="n"/>
-      <c r="F118" s="29">
+      <c r="A118" s="39" t="n"/>
+      <c r="B118" s="40" t="n"/>
+      <c r="C118" s="40" t="n"/>
+      <c r="D118" s="40" t="n"/>
+      <c r="E118" s="41" t="n"/>
+      <c r="F118" s="40">
         <f>IF(D118&lt;&gt;"Saída","",IF(E118&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B118,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -4375,12 +5134,12 @@
       <c r="H118" s="2" t="n"/>
     </row>
     <row r="119">
-      <c r="A119" s="28" t="n"/>
-      <c r="B119" s="29" t="n"/>
-      <c r="C119" s="29" t="n"/>
-      <c r="D119" s="29" t="n"/>
-      <c r="E119" s="30" t="n"/>
-      <c r="F119" s="29">
+      <c r="A119" s="39" t="n"/>
+      <c r="B119" s="40" t="n"/>
+      <c r="C119" s="40" t="n"/>
+      <c r="D119" s="40" t="n"/>
+      <c r="E119" s="41" t="n"/>
+      <c r="F119" s="40">
         <f>IF(D119&lt;&gt;"Saída","",IF(E119&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B119,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -4388,12 +5147,12 @@
       <c r="H119" s="2" t="n"/>
     </row>
     <row r="120">
-      <c r="A120" s="28" t="n"/>
-      <c r="B120" s="29" t="n"/>
-      <c r="C120" s="29" t="n"/>
-      <c r="D120" s="29" t="n"/>
-      <c r="E120" s="30" t="n"/>
-      <c r="F120" s="29">
+      <c r="A120" s="39" t="n"/>
+      <c r="B120" s="40" t="n"/>
+      <c r="C120" s="40" t="n"/>
+      <c r="D120" s="40" t="n"/>
+      <c r="E120" s="41" t="n"/>
+      <c r="F120" s="40">
         <f>IF(D120&lt;&gt;"Saída","",IF(E120&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B120,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -4401,12 +5160,12 @@
       <c r="H120" s="2" t="n"/>
     </row>
     <row r="121">
-      <c r="A121" s="28" t="n"/>
-      <c r="B121" s="29" t="n"/>
-      <c r="C121" s="29" t="n"/>
-      <c r="D121" s="29" t="n"/>
-      <c r="E121" s="30" t="n"/>
-      <c r="F121" s="29">
+      <c r="A121" s="39" t="n"/>
+      <c r="B121" s="40" t="n"/>
+      <c r="C121" s="40" t="n"/>
+      <c r="D121" s="40" t="n"/>
+      <c r="E121" s="41" t="n"/>
+      <c r="F121" s="40">
         <f>IF(D121&lt;&gt;"Saída","",IF(E121&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B121,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -4414,12 +5173,12 @@
       <c r="H121" s="2" t="n"/>
     </row>
     <row r="122">
-      <c r="A122" s="28" t="n"/>
-      <c r="B122" s="29" t="n"/>
-      <c r="C122" s="29" t="n"/>
-      <c r="D122" s="29" t="n"/>
-      <c r="E122" s="30" t="n"/>
-      <c r="F122" s="29">
+      <c r="A122" s="39" t="n"/>
+      <c r="B122" s="40" t="n"/>
+      <c r="C122" s="40" t="n"/>
+      <c r="D122" s="40" t="n"/>
+      <c r="E122" s="41" t="n"/>
+      <c r="F122" s="40">
         <f>IF(D122&lt;&gt;"Saída","",IF(E122&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B122,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -4427,12 +5186,12 @@
       <c r="H122" s="2" t="n"/>
     </row>
     <row r="123">
-      <c r="A123" s="28" t="n"/>
-      <c r="B123" s="29" t="n"/>
-      <c r="C123" s="29" t="n"/>
-      <c r="D123" s="29" t="n"/>
-      <c r="E123" s="30" t="n"/>
-      <c r="F123" s="29">
+      <c r="A123" s="39" t="n"/>
+      <c r="B123" s="40" t="n"/>
+      <c r="C123" s="40" t="n"/>
+      <c r="D123" s="40" t="n"/>
+      <c r="E123" s="41" t="n"/>
+      <c r="F123" s="40">
         <f>IF(D123&lt;&gt;"Saída","",IF(E123&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B123,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -4440,12 +5199,12 @@
       <c r="H123" s="2" t="n"/>
     </row>
     <row r="124">
-      <c r="A124" s="28" t="n"/>
-      <c r="B124" s="29" t="n"/>
-      <c r="C124" s="29" t="n"/>
-      <c r="D124" s="29" t="n"/>
-      <c r="E124" s="30" t="n"/>
-      <c r="F124" s="29">
+      <c r="A124" s="39" t="n"/>
+      <c r="B124" s="40" t="n"/>
+      <c r="C124" s="40" t="n"/>
+      <c r="D124" s="40" t="n"/>
+      <c r="E124" s="41" t="n"/>
+      <c r="F124" s="40">
         <f>IF(D124&lt;&gt;"Saída","",IF(E124&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B124,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -4453,12 +5212,12 @@
       <c r="H124" s="2" t="n"/>
     </row>
     <row r="125">
-      <c r="A125" s="28" t="n"/>
-      <c r="B125" s="29" t="n"/>
-      <c r="C125" s="29" t="n"/>
-      <c r="D125" s="29" t="n"/>
-      <c r="E125" s="30" t="n"/>
-      <c r="F125" s="29">
+      <c r="A125" s="39" t="n"/>
+      <c r="B125" s="40" t="n"/>
+      <c r="C125" s="40" t="n"/>
+      <c r="D125" s="40" t="n"/>
+      <c r="E125" s="41" t="n"/>
+      <c r="F125" s="40">
         <f>IF(D125&lt;&gt;"Saída","",IF(E125&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B125,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -4466,12 +5225,12 @@
       <c r="H125" s="2" t="n"/>
     </row>
     <row r="126">
-      <c r="A126" s="28" t="n"/>
-      <c r="B126" s="29" t="n"/>
-      <c r="C126" s="29" t="n"/>
-      <c r="D126" s="29" t="n"/>
-      <c r="E126" s="30" t="n"/>
-      <c r="F126" s="29">
+      <c r="A126" s="39" t="n"/>
+      <c r="B126" s="40" t="n"/>
+      <c r="C126" s="40" t="n"/>
+      <c r="D126" s="40" t="n"/>
+      <c r="E126" s="41" t="n"/>
+      <c r="F126" s="40">
         <f>IF(D126&lt;&gt;"Saída","",IF(E126&gt;SUMIF($D$6:$D$205,"Entrada",$E$6:$E$205)*IFERROR(VLOOKUP(B126,CONFIG!$A$4:$B$13,2,0),1),"⚠ acima do teto","ok"))</f>
         <v/>
       </c>
@@ -5225,7 +5984,7 @@
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <conditionalFormatting sqref="F6:F126">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="2">
       <formula>"⚠ acima do teto"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5319,12 +6078,12 @@
       <c r="H4" s="2" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="27" t="inlineStr">
+      <c r="A5" s="38" t="inlineStr">
         <is>
           <t>Aporte mensal (sobra)</t>
         </is>
       </c>
-      <c r="B5" s="31">
+      <c r="B5" s="42">
         <f>DASHBOARD!C10</f>
         <v/>
       </c>
@@ -5336,12 +6095,12 @@
       <c r="H5" s="2" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="27" t="inlineStr">
+      <c r="A6" s="38" t="inlineStr">
         <is>
           <t>Rendimento a.m.</t>
         </is>
       </c>
-      <c r="B6" s="32" t="n">
+      <c r="B6" s="43" t="n">
         <v>0.008</v>
       </c>
       <c r="C6" s="2" t="n"/>
@@ -5352,12 +6111,12 @@
       <c r="H6" s="2" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="27" t="inlineStr">
+      <c r="A7" s="38" t="inlineStr">
         <is>
           <t>Patrimônio inicial</t>
         </is>
       </c>
-      <c r="B7" s="33" t="n">
+      <c r="B7" s="44" t="n">
         <v>5000</v>
       </c>
       <c r="C7" s="2" t="n"/>
@@ -5396,10 +6155,10 @@
       <c r="H9" s="2" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="25" t="n">
+      <c r="A10" s="36" t="n">
         <v>1</v>
       </c>
-      <c r="B10" s="34">
+      <c r="B10" s="45">
         <f>$B$7*(1+$B$6)+$B$5</f>
         <v/>
       </c>
@@ -5411,10 +6170,10 @@
       <c r="H10" s="2" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="25" t="n">
+      <c r="A11" s="36" t="n">
         <v>2</v>
       </c>
-      <c r="B11" s="34">
+      <c r="B11" s="45">
         <f>B10*(1+$B$6)+$B$5</f>
         <v/>
       </c>
@@ -5426,10 +6185,10 @@
       <c r="H11" s="2" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="25" t="n">
+      <c r="A12" s="36" t="n">
         <v>3</v>
       </c>
-      <c r="B12" s="34">
+      <c r="B12" s="45">
         <f>B11*(1+$B$6)+$B$5</f>
         <v/>
       </c>
@@ -5441,10 +6200,10 @@
       <c r="H12" s="2" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="25" t="n">
+      <c r="A13" s="36" t="n">
         <v>4</v>
       </c>
-      <c r="B13" s="34">
+      <c r="B13" s="45">
         <f>B12*(1+$B$6)+$B$5</f>
         <v/>
       </c>
@@ -5456,10 +6215,10 @@
       <c r="H13" s="2" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="25" t="n">
+      <c r="A14" s="36" t="n">
         <v>5</v>
       </c>
-      <c r="B14" s="34">
+      <c r="B14" s="45">
         <f>B13*(1+$B$6)+$B$5</f>
         <v/>
       </c>
@@ -5471,10 +6230,10 @@
       <c r="H14" s="2" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="25" t="n">
+      <c r="A15" s="36" t="n">
         <v>6</v>
       </c>
-      <c r="B15" s="34">
+      <c r="B15" s="45">
         <f>B14*(1+$B$6)+$B$5</f>
         <v/>
       </c>
@@ -5486,10 +6245,10 @@
       <c r="H15" s="2" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="25" t="n">
+      <c r="A16" s="36" t="n">
         <v>7</v>
       </c>
-      <c r="B16" s="34">
+      <c r="B16" s="45">
         <f>B15*(1+$B$6)+$B$5</f>
         <v/>
       </c>
@@ -5501,10 +6260,10 @@
       <c r="H16" s="2" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="25" t="n">
+      <c r="A17" s="36" t="n">
         <v>8</v>
       </c>
-      <c r="B17" s="34">
+      <c r="B17" s="45">
         <f>B16*(1+$B$6)+$B$5</f>
         <v/>
       </c>
@@ -5516,10 +6275,10 @@
       <c r="H17" s="2" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="25" t="n">
+      <c r="A18" s="36" t="n">
         <v>9</v>
       </c>
-      <c r="B18" s="34">
+      <c r="B18" s="45">
         <f>B17*(1+$B$6)+$B$5</f>
         <v/>
       </c>
@@ -5531,10 +6290,10 @@
       <c r="H18" s="2" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="25" t="n">
+      <c r="A19" s="36" t="n">
         <v>10</v>
       </c>
-      <c r="B19" s="34">
+      <c r="B19" s="45">
         <f>B18*(1+$B$6)+$B$5</f>
         <v/>
       </c>
@@ -5546,10 +6305,10 @@
       <c r="H19" s="2" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="25" t="n">
+      <c r="A20" s="36" t="n">
         <v>11</v>
       </c>
-      <c r="B20" s="34">
+      <c r="B20" s="45">
         <f>B19*(1+$B$6)+$B$5</f>
         <v/>
       </c>
@@ -5561,10 +6320,10 @@
       <c r="H20" s="2" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="25" t="n">
+      <c r="A21" s="36" t="n">
         <v>12</v>
       </c>
-      <c r="B21" s="34">
+      <c r="B21" s="45">
         <f>B20*(1+$B$6)+$B$5</f>
         <v/>
       </c>

</xml_diff>